<commit_message>
fix: Update homepage links 404 audit report and dashboard for Beta
</commit_message>
<xml_diff>
--- a/Homepage_Links_Navigation_Report.xlsx
+++ b/Homepage_Links_Navigation_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3243" uniqueCount="690">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3111" uniqueCount="680">
   <si>
     <t>ID</t>
   </si>
@@ -1480,10 +1480,7 @@
     <t>Online Furniture Shopping Website</t>
   </si>
   <si>
-    <t>https://beta.teamwoodenstreet.com/freedom-sale</t>
-  </si>
-  <si>
-    <t>FAIL (404 Not Found)</t>
+    <t>https://beta.teamwoodenstreet.com/festive-sale</t>
   </si>
   <si>
     <t>Buy Furniture Online in India</t>
@@ -1501,7 +1498,7 @@
     <t>SOFAS</t>
   </si>
   <si>
-    <t>https://beta.teamwoodenstreet.com/all-sofa</t>
+    <t>https://beta.teamwoodenstreet.com/sofa</t>
   </si>
   <si>
     <t>BEDS</t>
@@ -1612,9 +1609,6 @@
     <t>Wooden Street Sofa</t>
   </si>
   <si>
-    <t>https://beta.teamwoodenstreet.com/sofa</t>
-  </si>
-  <si>
     <t>woodenstreet - TV Units</t>
   </si>
   <si>
@@ -1630,6 +1624,9 @@
     <t>woodenstreet - All Study Tables</t>
   </si>
   <si>
+    <t>woodenstreet - All Sofa cum bed</t>
+  </si>
+  <si>
     <t>woodenstreet - All Coffee &amp; Centre Table</t>
   </si>
   <si>
@@ -1645,202 +1642,175 @@
     <t>SHOP BEDROOM</t>
   </si>
   <si>
-    <t>WoodenStreet Media Partners</t>
+    <t>solid wood furniture</t>
+  </si>
+  <si>
+    <t>https://beta.teamwoodenstreet.com/solid-wood-furniture</t>
+  </si>
+  <si>
+    <t>sofa set</t>
+  </si>
+  <si>
+    <t>recliner</t>
+  </si>
+  <si>
+    <t>coffee table for living room</t>
+  </si>
+  <si>
+    <t>carpets</t>
+  </si>
+  <si>
+    <t>TV units</t>
+  </si>
+  <si>
+    <t>single bed</t>
+  </si>
+  <si>
+    <t>double bed</t>
+  </si>
+  <si>
+    <t>divan bed</t>
+  </si>
+  <si>
+    <t>dressing table</t>
+  </si>
+  <si>
+    <t>bunk bed</t>
+  </si>
+  <si>
+    <t>https://beta.teamwoodenstreet.com/bunk-beds</t>
+  </si>
+  <si>
+    <t>Wardrobe</t>
+  </si>
+  <si>
+    <t>buy a bed online</t>
+  </si>
+  <si>
+    <t>mattresses</t>
+  </si>
+  <si>
+    <t>cushions</t>
+  </si>
+  <si>
+    <t>https://beta.teamwoodenstreet.com/cushions</t>
+  </si>
+  <si>
+    <t>dining table</t>
+  </si>
+  <si>
+    <t>dining chairs</t>
+  </si>
+  <si>
+    <t>kitchen cabinets</t>
+  </si>
+  <si>
+    <t>crockery units</t>
+  </si>
+  <si>
+    <t>folding dining tables</t>
+  </si>
+  <si>
+    <t>foldable study tables</t>
+  </si>
+  <si>
+    <t>bookshelves</t>
+  </si>
+  <si>
+    <t>computer tables</t>
+  </si>
+  <si>
+    <t>study table</t>
+  </si>
+  <si>
+    <t>study chairs</t>
+  </si>
+  <si>
+    <t>kids bed</t>
+  </si>
+  <si>
+    <t>office chairs</t>
+  </si>
+  <si>
+    <t>office tables</t>
+  </si>
+  <si>
+    <t>computer chair</t>
+  </si>
+  <si>
+    <t>https://beta.teamwoodenstreet.com/computer-chairs</t>
+  </si>
+  <si>
+    <t>executive chair</t>
+  </si>
+  <si>
+    <t>ergonomic chair</t>
+  </si>
+  <si>
+    <t>https://beta.teamwoodenstreet.com/ergonomic-chair</t>
+  </si>
+  <si>
+    <t>revolving chair</t>
+  </si>
+  <si>
+    <t>https://beta.teamwoodenstreet.com/revolving-chair</t>
+  </si>
+  <si>
+    <t>office sofa</t>
+  </si>
+  <si>
+    <t>home decor</t>
+  </si>
+  <si>
+    <t>wall mirrors,</t>
+  </si>
+  <si>
+    <t>gifts</t>
+  </si>
+  <si>
+    <t>https://beta.teamwoodenstreet.com/gift</t>
+  </si>
+  <si>
+    <t>shoe rack</t>
+  </si>
+  <si>
+    <t>foldable mattress</t>
+  </si>
+  <si>
+    <t>latex mattress</t>
+  </si>
+  <si>
+    <t>About Us</t>
+  </si>
+  <si>
+    <t>https://beta.teamwoodenstreet.com/about-us</t>
+  </si>
+  <si>
+    <t>Career</t>
+  </si>
+  <si>
+    <t>https://beta.teamwoodenstreet.com/careers</t>
+  </si>
+  <si>
+    <t>Media</t>
   </si>
   <si>
     <t>https://beta.teamwoodenstreet.com/media</t>
   </si>
   <si>
-    <t>[Banner / Image Link]</t>
-  </si>
-  <si>
-    <t>View Product</t>
-  </si>
-  <si>
-    <t>https://www.woodenstreet.com/product/lorenz-3-seater-sofa-velvet-graphite-grey</t>
-  </si>
-  <si>
-    <t>https://www.woodenstreet.com/product/reveka-chest-of-drawer-walnut-finish</t>
-  </si>
-  <si>
-    <t>https://www.woodenstreet.com/product/vedic-3-seater-sofa-with-cane-and-brass-detail-teak-finish-jade-ivory</t>
-  </si>
-  <si>
-    <t>https://www.woodenstreet.com/product/travolta-divan-walnut-finish</t>
-  </si>
-  <si>
-    <t>https://www.woodenstreet.com/product/reveka-chest-of-drawer-honey-finish</t>
-  </si>
-  <si>
-    <t>View All</t>
+    <t>Blog</t>
+  </si>
+  <si>
+    <t>https://www.woodenstreet.com/blog/</t>
+  </si>
+  <si>
+    <t>Our Stores</t>
+  </si>
+  <si>
+    <t>Customer Stories</t>
   </si>
   <si>
     <t>https://beta.teamwoodenstreet.com/customer-stories</t>
-  </si>
-  <si>
-    <t>solid wood furniture</t>
-  </si>
-  <si>
-    <t>https://beta.teamwoodenstreet.com/solid-wood-furniture</t>
-  </si>
-  <si>
-    <t>sofa set</t>
-  </si>
-  <si>
-    <t>recliner</t>
-  </si>
-  <si>
-    <t>coffee table for living room</t>
-  </si>
-  <si>
-    <t>carpets</t>
-  </si>
-  <si>
-    <t>TV units</t>
-  </si>
-  <si>
-    <t>single bed</t>
-  </si>
-  <si>
-    <t>double bed</t>
-  </si>
-  <si>
-    <t>divan bed</t>
-  </si>
-  <si>
-    <t>dressing table</t>
-  </si>
-  <si>
-    <t>bunk bed</t>
-  </si>
-  <si>
-    <t>https://beta.teamwoodenstreet.com/bunk-beds</t>
-  </si>
-  <si>
-    <t>Wardrobe</t>
-  </si>
-  <si>
-    <t>buy a bed online</t>
-  </si>
-  <si>
-    <t>mattresses</t>
-  </si>
-  <si>
-    <t>cushions</t>
-  </si>
-  <si>
-    <t>https://beta.teamwoodenstreet.com/cushions</t>
-  </si>
-  <si>
-    <t>dining table</t>
-  </si>
-  <si>
-    <t>dining chairs</t>
-  </si>
-  <si>
-    <t>kitchen cabinets</t>
-  </si>
-  <si>
-    <t>crockery units</t>
-  </si>
-  <si>
-    <t>folding dining tables</t>
-  </si>
-  <si>
-    <t>foldable study tables</t>
-  </si>
-  <si>
-    <t>bookshelves</t>
-  </si>
-  <si>
-    <t>computer tables</t>
-  </si>
-  <si>
-    <t>study table</t>
-  </si>
-  <si>
-    <t>study chairs</t>
-  </si>
-  <si>
-    <t>kids bed</t>
-  </si>
-  <si>
-    <t>office chairs</t>
-  </si>
-  <si>
-    <t>office tables</t>
-  </si>
-  <si>
-    <t>computer chair</t>
-  </si>
-  <si>
-    <t>https://beta.teamwoodenstreet.com/computer-chairs</t>
-  </si>
-  <si>
-    <t>executive chair</t>
-  </si>
-  <si>
-    <t>ergonomic chair</t>
-  </si>
-  <si>
-    <t>https://beta.teamwoodenstreet.com/ergonomic-chair</t>
-  </si>
-  <si>
-    <t>revolving chair</t>
-  </si>
-  <si>
-    <t>https://beta.teamwoodenstreet.com/revolving-chair</t>
-  </si>
-  <si>
-    <t>office sofa</t>
-  </si>
-  <si>
-    <t>home decor</t>
-  </si>
-  <si>
-    <t>wall mirrors,</t>
-  </si>
-  <si>
-    <t>gifts</t>
-  </si>
-  <si>
-    <t>https://beta.teamwoodenstreet.com/gift</t>
-  </si>
-  <si>
-    <t>shoe rack</t>
-  </si>
-  <si>
-    <t>foldable mattress</t>
-  </si>
-  <si>
-    <t>latex mattress</t>
-  </si>
-  <si>
-    <t>About Us</t>
-  </si>
-  <si>
-    <t>https://beta.teamwoodenstreet.com/about-us</t>
-  </si>
-  <si>
-    <t>Career</t>
-  </si>
-  <si>
-    <t>https://beta.teamwoodenstreet.com/careers</t>
-  </si>
-  <si>
-    <t>Media</t>
-  </si>
-  <si>
-    <t>Blog</t>
-  </si>
-  <si>
-    <t>https://www.woodenstreet.com/blog/</t>
-  </si>
-  <si>
-    <t>Our Stores</t>
-  </si>
-  <si>
-    <t>Customer Stories</t>
   </si>
   <si>
     <t>Investor Relations</t>
@@ -2497,7 +2467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H540"/>
+  <dimension ref="A1:H518"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -11479,30 +11449,30 @@
         <v>11</v>
       </c>
     </row>
-    <row r="346" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A346" s="5">
+    <row r="346" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A346">
         <v>345</v>
       </c>
-      <c r="B346" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C346" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D346" s="5" t="s">
+      <c r="B346" t="s">
+        <v>8</v>
+      </c>
+      <c r="C346" t="s">
+        <v>9</v>
+      </c>
+      <c r="D346" t="s">
         <v>488</v>
       </c>
-      <c r="E346" s="5" t="s">
+      <c r="E346" t="s">
         <v>489</v>
       </c>
-      <c r="F346" s="5" t="s">
+      <c r="F346" t="s">
         <v>489</v>
       </c>
-      <c r="G346" s="6">
-        <v>404</v>
-      </c>
-      <c r="H346" s="6" t="s">
-        <v>490</v>
+      <c r="G346">
+        <v>200</v>
+      </c>
+      <c r="H346" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="347" spans="1:8" x14ac:dyDescent="0.25">
@@ -11516,7 +11486,7 @@
         <v>9</v>
       </c>
       <c r="D347" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E347" t="s">
         <v>181</v>
@@ -11542,7 +11512,7 @@
         <v>9</v>
       </c>
       <c r="D348" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E348" t="s">
         <v>288</v>
@@ -11568,7 +11538,7 @@
         <v>9</v>
       </c>
       <c r="D349" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="E349" t="s">
         <v>32</v>
@@ -11594,7 +11564,7 @@
         <v>9</v>
       </c>
       <c r="D350" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E350" t="s">
         <v>30</v>
@@ -11620,7 +11590,7 @@
         <v>9</v>
       </c>
       <c r="D351" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="E351" t="s">
         <v>40</v>
@@ -11646,7 +11616,7 @@
         <v>9</v>
       </c>
       <c r="D352" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="E352" t="s">
         <v>370</v>
@@ -11661,30 +11631,30 @@
         <v>11</v>
       </c>
     </row>
-    <row r="353" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A353" s="5">
+    <row r="353" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A353">
         <v>352</v>
       </c>
-      <c r="B353" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C353" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D353" s="5" t="s">
+      <c r="B353" t="s">
+        <v>8</v>
+      </c>
+      <c r="C353" t="s">
+        <v>9</v>
+      </c>
+      <c r="D353" t="s">
+        <v>494</v>
+      </c>
+      <c r="E353" t="s">
         <v>495</v>
       </c>
-      <c r="E353" s="5" t="s">
-        <v>496</v>
-      </c>
-      <c r="F353" s="5" t="s">
-        <v>496</v>
-      </c>
-      <c r="G353" s="6">
-        <v>404</v>
-      </c>
-      <c r="H353" s="6" t="s">
-        <v>490</v>
+      <c r="F353" t="s">
+        <v>495</v>
+      </c>
+      <c r="G353">
+        <v>200</v>
+      </c>
+      <c r="H353" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="354" spans="1:8" x14ac:dyDescent="0.25">
@@ -11698,7 +11668,7 @@
         <v>9</v>
       </c>
       <c r="D354" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E354" t="s">
         <v>181</v>
@@ -11724,13 +11694,13 @@
         <v>9</v>
       </c>
       <c r="D355" t="s">
+        <v>497</v>
+      </c>
+      <c r="E355" t="s">
         <v>498</v>
       </c>
-      <c r="E355" t="s">
-        <v>499</v>
-      </c>
       <c r="F355" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="G355">
         <v>200</v>
@@ -11750,13 +11720,13 @@
         <v>9</v>
       </c>
       <c r="D356" t="s">
+        <v>499</v>
+      </c>
+      <c r="E356" t="s">
         <v>500</v>
       </c>
-      <c r="E356" t="s">
-        <v>501</v>
-      </c>
       <c r="F356" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G356">
         <v>200</v>
@@ -11776,7 +11746,7 @@
         <v>9</v>
       </c>
       <c r="D357" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="E357" t="s">
         <v>44</v>
@@ -11802,7 +11772,7 @@
         <v>9</v>
       </c>
       <c r="D358" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="E358" t="s">
         <v>70</v>
@@ -11828,13 +11798,13 @@
         <v>9</v>
       </c>
       <c r="D359" t="s">
+        <v>503</v>
+      </c>
+      <c r="E359" t="s">
         <v>504</v>
       </c>
-      <c r="E359" t="s">
-        <v>505</v>
-      </c>
       <c r="F359" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="G359">
         <v>200</v>
@@ -11854,7 +11824,7 @@
         <v>9</v>
       </c>
       <c r="D360" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="E360" t="s">
         <v>370</v>
@@ -11880,7 +11850,7 @@
         <v>9</v>
       </c>
       <c r="D361" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="E361" t="s">
         <v>207</v>
@@ -11906,13 +11876,13 @@
         <v>9</v>
       </c>
       <c r="D362" t="s">
+        <v>507</v>
+      </c>
+      <c r="E362" t="s">
         <v>508</v>
       </c>
-      <c r="E362" t="s">
-        <v>509</v>
-      </c>
       <c r="F362" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="G362">
         <v>200</v>
@@ -11932,7 +11902,7 @@
         <v>9</v>
       </c>
       <c r="D363" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="E363" t="s">
         <v>52</v>
@@ -11958,7 +11928,7 @@
         <v>9</v>
       </c>
       <c r="D364" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="E364" t="s">
         <v>232</v>
@@ -11984,13 +11954,13 @@
         <v>9</v>
       </c>
       <c r="D365" t="s">
+        <v>510</v>
+      </c>
+      <c r="E365" t="s">
         <v>511</v>
       </c>
-      <c r="E365" t="s">
-        <v>512</v>
-      </c>
       <c r="F365" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G365">
         <v>200</v>
@@ -12013,10 +11983,10 @@
         <v>10</v>
       </c>
       <c r="E366" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="F366" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="G366">
         <v>200</v>
@@ -12036,7 +12006,7 @@
         <v>9</v>
       </c>
       <c r="D367" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="E367" t="s">
         <v>114</v>
@@ -12062,7 +12032,7 @@
         <v>9</v>
       </c>
       <c r="D368" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="E368" t="s">
         <v>177</v>
@@ -12088,7 +12058,7 @@
         <v>9</v>
       </c>
       <c r="D369" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="E369" t="s">
         <v>283</v>
@@ -12114,7 +12084,7 @@
         <v>9</v>
       </c>
       <c r="D370" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="E370" t="s">
         <v>367</v>
@@ -12140,13 +12110,13 @@
         <v>9</v>
       </c>
       <c r="D371" t="s">
+        <v>517</v>
+      </c>
+      <c r="E371" t="s">
         <v>518</v>
       </c>
-      <c r="E371" t="s">
-        <v>519</v>
-      </c>
       <c r="F371" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="G371">
         <v>200</v>
@@ -12166,13 +12136,13 @@
         <v>9</v>
       </c>
       <c r="D372" t="s">
+        <v>519</v>
+      </c>
+      <c r="E372" t="s">
         <v>520</v>
       </c>
-      <c r="E372" t="s">
-        <v>521</v>
-      </c>
       <c r="F372" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="G372">
         <v>200</v>
@@ -12192,13 +12162,13 @@
         <v>9</v>
       </c>
       <c r="D373" t="s">
+        <v>521</v>
+      </c>
+      <c r="E373" t="s">
         <v>522</v>
       </c>
-      <c r="E373" t="s">
-        <v>523</v>
-      </c>
       <c r="F373" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="G373">
         <v>200</v>
@@ -12218,13 +12188,13 @@
         <v>9</v>
       </c>
       <c r="D374" t="s">
+        <v>523</v>
+      </c>
+      <c r="E374" t="s">
         <v>524</v>
       </c>
-      <c r="E374" t="s">
-        <v>525</v>
-      </c>
       <c r="F374" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G374">
         <v>200</v>
@@ -12244,13 +12214,13 @@
         <v>9</v>
       </c>
       <c r="D375" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="E375" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="F375" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="G375">
         <v>200</v>
@@ -12270,13 +12240,13 @@
         <v>9</v>
       </c>
       <c r="D376" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E376" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="F376" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="G376">
         <v>200</v>
@@ -12296,13 +12266,13 @@
         <v>9</v>
       </c>
       <c r="D377" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="E377" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="F377" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="G377">
         <v>200</v>
@@ -12322,13 +12292,13 @@
         <v>9</v>
       </c>
       <c r="D378" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="E378" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="F378" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G378">
         <v>200</v>
@@ -12348,13 +12318,13 @@
         <v>9</v>
       </c>
       <c r="D379" t="s">
+        <v>529</v>
+      </c>
+      <c r="E379" t="s">
         <v>530</v>
       </c>
-      <c r="E379" t="s">
-        <v>531</v>
-      </c>
       <c r="F379" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="G379">
         <v>200</v>
@@ -12374,13 +12344,13 @@
         <v>9</v>
       </c>
       <c r="D380" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="E380" t="s">
-        <v>533</v>
+        <v>495</v>
       </c>
       <c r="F380" t="s">
-        <v>533</v>
+        <v>495</v>
       </c>
       <c r="G380">
         <v>200</v>
@@ -12400,7 +12370,7 @@
         <v>9</v>
       </c>
       <c r="D381" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="E381" t="s">
         <v>44</v>
@@ -12426,7 +12396,7 @@
         <v>9</v>
       </c>
       <c r="D382" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="E382" t="s">
         <v>385</v>
@@ -12452,13 +12422,13 @@
         <v>9</v>
       </c>
       <c r="D383" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="E383" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="F383" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="G383">
         <v>200</v>
@@ -12478,7 +12448,7 @@
         <v>9</v>
       </c>
       <c r="D384" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="E384" t="s">
         <v>370</v>
@@ -12504,7 +12474,7 @@
         <v>9</v>
       </c>
       <c r="D385" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="E385" t="s">
         <v>70</v>
@@ -12530,13 +12500,13 @@
         <v>9</v>
       </c>
       <c r="D386" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="E386" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="F386" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="G386">
         <v>200</v>
@@ -12556,7 +12526,7 @@
         <v>9</v>
       </c>
       <c r="D387" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="E387" t="s">
         <v>288</v>
@@ -12582,7 +12552,7 @@
         <v>9</v>
       </c>
       <c r="D388" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="E388" t="s">
         <v>283</v>
@@ -12608,7 +12578,7 @@
         <v>9</v>
       </c>
       <c r="D389" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="E389" t="s">
         <v>283</v>
@@ -12634,7 +12604,7 @@
         <v>9</v>
       </c>
       <c r="D390" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="E390" t="s">
         <v>288</v>
@@ -12660,7 +12630,7 @@
         <v>9</v>
       </c>
       <c r="D391" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="E391" t="s">
         <v>283</v>
@@ -12686,7 +12656,7 @@
         <v>9</v>
       </c>
       <c r="D392" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="E392" t="s">
         <v>283</v>
@@ -12712,7 +12682,7 @@
         <v>9</v>
       </c>
       <c r="D393" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E393" t="s">
         <v>181</v>
@@ -12738,7 +12708,7 @@
         <v>9</v>
       </c>
       <c r="D394" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E394" t="s">
         <v>177</v>
@@ -12764,7 +12734,7 @@
         <v>9</v>
       </c>
       <c r="D395" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="E395" t="s">
         <v>177</v>
@@ -12790,7 +12760,7 @@
         <v>9</v>
       </c>
       <c r="D396" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E396" t="s">
         <v>181</v>
@@ -12816,7 +12786,7 @@
         <v>9</v>
       </c>
       <c r="D397" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E397" t="s">
         <v>177</v>
@@ -12842,7 +12812,7 @@
         <v>9</v>
       </c>
       <c r="D398" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="E398" t="s">
         <v>177</v>
@@ -12868,13 +12838,13 @@
         <v>9</v>
       </c>
       <c r="D399" t="s">
+        <v>543</v>
+      </c>
+      <c r="E399" t="s">
         <v>544</v>
       </c>
-      <c r="E399" t="s">
-        <v>545</v>
-      </c>
       <c r="F399" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="G399">
         <v>200</v>
@@ -12894,13 +12864,13 @@
         <v>9</v>
       </c>
       <c r="D400" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E400" t="s">
-        <v>545</v>
+        <v>61</v>
       </c>
       <c r="F400" t="s">
-        <v>545</v>
+        <v>61</v>
       </c>
       <c r="G400">
         <v>200</v>
@@ -12920,13 +12890,13 @@
         <v>9</v>
       </c>
       <c r="D401" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="E401" t="s">
-        <v>545</v>
+        <v>88</v>
       </c>
       <c r="F401" t="s">
-        <v>545</v>
+        <v>88</v>
       </c>
       <c r="G401">
         <v>200</v>
@@ -12946,13 +12916,13 @@
         <v>9</v>
       </c>
       <c r="D402" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="E402" t="s">
-        <v>545</v>
+        <v>30</v>
       </c>
       <c r="F402" t="s">
-        <v>545</v>
+        <v>30</v>
       </c>
       <c r="G402">
         <v>200</v>
@@ -12972,13 +12942,13 @@
         <v>9</v>
       </c>
       <c r="D403" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="E403" t="s">
-        <v>545</v>
+        <v>171</v>
       </c>
       <c r="F403" t="s">
-        <v>545</v>
+        <v>171</v>
       </c>
       <c r="G403">
         <v>200</v>
@@ -12998,13 +12968,13 @@
         <v>9</v>
       </c>
       <c r="D404" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="E404" t="s">
-        <v>545</v>
+        <v>44</v>
       </c>
       <c r="F404" t="s">
-        <v>545</v>
+        <v>44</v>
       </c>
       <c r="G404">
         <v>200</v>
@@ -13024,13 +12994,13 @@
         <v>9</v>
       </c>
       <c r="D405" t="s">
-        <v>546</v>
+        <v>81</v>
       </c>
       <c r="E405" t="s">
-        <v>545</v>
+        <v>32</v>
       </c>
       <c r="F405" t="s">
-        <v>545</v>
+        <v>32</v>
       </c>
       <c r="G405">
         <v>200</v>
@@ -13050,13 +13020,13 @@
         <v>9</v>
       </c>
       <c r="D406" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="E406" t="s">
-        <v>545</v>
+        <v>201</v>
       </c>
       <c r="F406" t="s">
-        <v>545</v>
+        <v>201</v>
       </c>
       <c r="G406">
         <v>200</v>
@@ -13076,13 +13046,13 @@
         <v>9</v>
       </c>
       <c r="D407" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="E407" t="s">
-        <v>545</v>
+        <v>199</v>
       </c>
       <c r="F407" t="s">
-        <v>545</v>
+        <v>199</v>
       </c>
       <c r="G407">
         <v>200</v>
@@ -13102,13 +13072,13 @@
         <v>9</v>
       </c>
       <c r="D408" t="s">
-        <v>544</v>
+        <v>552</v>
       </c>
       <c r="E408" t="s">
-        <v>545</v>
+        <v>80</v>
       </c>
       <c r="F408" t="s">
-        <v>545</v>
+        <v>80</v>
       </c>
       <c r="G408">
         <v>200</v>
@@ -13128,13 +13098,13 @@
         <v>9</v>
       </c>
       <c r="D409" t="s">
-        <v>544</v>
+        <v>553</v>
       </c>
       <c r="E409" t="s">
-        <v>545</v>
+        <v>226</v>
       </c>
       <c r="F409" t="s">
-        <v>545</v>
+        <v>226</v>
       </c>
       <c r="G409">
         <v>200</v>
@@ -13154,13 +13124,13 @@
         <v>9</v>
       </c>
       <c r="D410" t="s">
-        <v>544</v>
+        <v>554</v>
       </c>
       <c r="E410" t="s">
-        <v>545</v>
+        <v>555</v>
       </c>
       <c r="F410" t="s">
-        <v>545</v>
+        <v>555</v>
       </c>
       <c r="G410">
         <v>200</v>
@@ -13180,13 +13150,13 @@
         <v>9</v>
       </c>
       <c r="D411" t="s">
-        <v>546</v>
+        <v>556</v>
       </c>
       <c r="E411" t="s">
-        <v>545</v>
+        <v>205</v>
       </c>
       <c r="F411" t="s">
-        <v>545</v>
+        <v>205</v>
       </c>
       <c r="G411">
         <v>200</v>
@@ -13206,13 +13176,13 @@
         <v>9</v>
       </c>
       <c r="D412" t="s">
-        <v>546</v>
+        <v>557</v>
       </c>
       <c r="E412" t="s">
-        <v>545</v>
+        <v>179</v>
       </c>
       <c r="F412" t="s">
-        <v>545</v>
+        <v>179</v>
       </c>
       <c r="G412">
         <v>200</v>
@@ -13232,13 +13202,13 @@
         <v>9</v>
       </c>
       <c r="D413" t="s">
-        <v>546</v>
+        <v>558</v>
       </c>
       <c r="E413" t="s">
-        <v>545</v>
+        <v>232</v>
       </c>
       <c r="F413" t="s">
-        <v>545</v>
+        <v>232</v>
       </c>
       <c r="G413">
         <v>200</v>
@@ -13258,13 +13228,13 @@
         <v>9</v>
       </c>
       <c r="D414" t="s">
-        <v>546</v>
+        <v>559</v>
       </c>
       <c r="E414" t="s">
-        <v>545</v>
+        <v>560</v>
       </c>
       <c r="F414" t="s">
-        <v>545</v>
+        <v>560</v>
       </c>
       <c r="G414">
         <v>200</v>
@@ -13284,13 +13254,13 @@
         <v>9</v>
       </c>
       <c r="D415" t="s">
-        <v>547</v>
+        <v>561</v>
       </c>
       <c r="E415" t="s">
-        <v>548</v>
+        <v>312</v>
       </c>
       <c r="F415" t="s">
-        <v>548</v>
+        <v>312</v>
       </c>
       <c r="G415">
         <v>200</v>
@@ -13310,13 +13280,13 @@
         <v>9</v>
       </c>
       <c r="D416" t="s">
-        <v>547</v>
+        <v>562</v>
       </c>
       <c r="E416" t="s">
-        <v>549</v>
+        <v>304</v>
       </c>
       <c r="F416" t="s">
-        <v>549</v>
+        <v>304</v>
       </c>
       <c r="G416">
         <v>200</v>
@@ -13336,13 +13306,13 @@
         <v>9</v>
       </c>
       <c r="D417" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="E417" t="s">
-        <v>550</v>
+        <v>323</v>
       </c>
       <c r="F417" t="s">
-        <v>550</v>
+        <v>323</v>
       </c>
       <c r="G417">
         <v>200</v>
@@ -13362,13 +13332,13 @@
         <v>9</v>
       </c>
       <c r="D418" t="s">
-        <v>547</v>
+        <v>564</v>
       </c>
       <c r="E418" t="s">
-        <v>551</v>
+        <v>361</v>
       </c>
       <c r="F418" t="s">
-        <v>551</v>
+        <v>361</v>
       </c>
       <c r="G418">
         <v>200</v>
@@ -13388,13 +13358,13 @@
         <v>9</v>
       </c>
       <c r="D419" t="s">
-        <v>547</v>
+        <v>565</v>
       </c>
       <c r="E419" t="s">
-        <v>552</v>
+        <v>296</v>
       </c>
       <c r="F419" t="s">
-        <v>552</v>
+        <v>296</v>
       </c>
       <c r="G419">
         <v>200</v>
@@ -13414,13 +13384,13 @@
         <v>9</v>
       </c>
       <c r="D420" t="s">
-        <v>553</v>
+        <v>566</v>
       </c>
       <c r="E420" t="s">
-        <v>554</v>
+        <v>374</v>
       </c>
       <c r="F420" t="s">
-        <v>554</v>
+        <v>374</v>
       </c>
       <c r="G420">
         <v>200</v>
@@ -13440,13 +13410,13 @@
         <v>9</v>
       </c>
       <c r="D421" t="s">
-        <v>555</v>
+        <v>567</v>
       </c>
       <c r="E421" t="s">
-        <v>556</v>
+        <v>153</v>
       </c>
       <c r="F421" t="s">
-        <v>556</v>
+        <v>153</v>
       </c>
       <c r="G421">
         <v>200</v>
@@ -13466,13 +13436,13 @@
         <v>9</v>
       </c>
       <c r="D422" t="s">
-        <v>557</v>
+        <v>568</v>
       </c>
       <c r="E422" t="s">
-        <v>61</v>
+        <v>372</v>
       </c>
       <c r="F422" t="s">
-        <v>61</v>
+        <v>372</v>
       </c>
       <c r="G422">
         <v>200</v>
@@ -13492,13 +13462,13 @@
         <v>9</v>
       </c>
       <c r="D423" t="s">
-        <v>558</v>
+        <v>569</v>
       </c>
       <c r="E423" t="s">
-        <v>88</v>
+        <v>368</v>
       </c>
       <c r="F423" t="s">
-        <v>88</v>
+        <v>368</v>
       </c>
       <c r="G423">
         <v>200</v>
@@ -13518,13 +13488,13 @@
         <v>9</v>
       </c>
       <c r="D424" t="s">
-        <v>559</v>
+        <v>570</v>
       </c>
       <c r="E424" t="s">
-        <v>30</v>
+        <v>387</v>
       </c>
       <c r="F424" t="s">
-        <v>30</v>
+        <v>387</v>
       </c>
       <c r="G424">
         <v>200</v>
@@ -13544,13 +13514,13 @@
         <v>9</v>
       </c>
       <c r="D425" t="s">
-        <v>560</v>
+        <v>571</v>
       </c>
       <c r="E425" t="s">
-        <v>171</v>
+        <v>193</v>
       </c>
       <c r="F425" t="s">
-        <v>171</v>
+        <v>193</v>
       </c>
       <c r="G425">
         <v>200</v>
@@ -13570,13 +13540,13 @@
         <v>9</v>
       </c>
       <c r="D426" t="s">
-        <v>561</v>
+        <v>572</v>
       </c>
       <c r="E426" t="s">
-        <v>44</v>
+        <v>385</v>
       </c>
       <c r="F426" t="s">
-        <v>44</v>
+        <v>385</v>
       </c>
       <c r="G426">
         <v>200</v>
@@ -13596,13 +13566,13 @@
         <v>9</v>
       </c>
       <c r="D427" t="s">
-        <v>81</v>
+        <v>573</v>
       </c>
       <c r="E427" t="s">
-        <v>32</v>
+        <v>382</v>
       </c>
       <c r="F427" t="s">
-        <v>32</v>
+        <v>382</v>
       </c>
       <c r="G427">
         <v>200</v>
@@ -13622,13 +13592,13 @@
         <v>9</v>
       </c>
       <c r="D428" t="s">
-        <v>562</v>
+        <v>574</v>
       </c>
       <c r="E428" t="s">
-        <v>201</v>
+        <v>575</v>
       </c>
       <c r="F428" t="s">
-        <v>201</v>
+        <v>575</v>
       </c>
       <c r="G428">
         <v>200</v>
@@ -13648,13 +13618,13 @@
         <v>9</v>
       </c>
       <c r="D429" t="s">
-        <v>563</v>
+        <v>576</v>
       </c>
       <c r="E429" t="s">
-        <v>199</v>
+        <v>391</v>
       </c>
       <c r="F429" t="s">
-        <v>199</v>
+        <v>391</v>
       </c>
       <c r="G429">
         <v>200</v>
@@ -13674,13 +13644,13 @@
         <v>9</v>
       </c>
       <c r="D430" t="s">
-        <v>564</v>
+        <v>577</v>
       </c>
       <c r="E430" t="s">
-        <v>80</v>
+        <v>578</v>
       </c>
       <c r="F430" t="s">
-        <v>80</v>
+        <v>578</v>
       </c>
       <c r="G430">
         <v>200</v>
@@ -13700,13 +13670,13 @@
         <v>9</v>
       </c>
       <c r="D431" t="s">
-        <v>565</v>
+        <v>579</v>
       </c>
       <c r="E431" t="s">
-        <v>226</v>
+        <v>580</v>
       </c>
       <c r="F431" t="s">
-        <v>226</v>
+        <v>580</v>
       </c>
       <c r="G431">
         <v>200</v>
@@ -13726,13 +13696,13 @@
         <v>9</v>
       </c>
       <c r="D432" t="s">
-        <v>566</v>
+        <v>581</v>
       </c>
       <c r="E432" t="s">
-        <v>567</v>
+        <v>395</v>
       </c>
       <c r="F432" t="s">
-        <v>567</v>
+        <v>395</v>
       </c>
       <c r="G432">
         <v>200</v>
@@ -13752,13 +13722,13 @@
         <v>9</v>
       </c>
       <c r="D433" t="s">
-        <v>568</v>
+        <v>582</v>
       </c>
       <c r="E433" t="s">
-        <v>205</v>
+        <v>46</v>
       </c>
       <c r="F433" t="s">
-        <v>205</v>
+        <v>46</v>
       </c>
       <c r="G433">
         <v>200</v>
@@ -13778,13 +13748,13 @@
         <v>9</v>
       </c>
       <c r="D434" t="s">
-        <v>569</v>
+        <v>583</v>
       </c>
       <c r="E434" t="s">
-        <v>179</v>
+        <v>429</v>
       </c>
       <c r="F434" t="s">
-        <v>179</v>
+        <v>429</v>
       </c>
       <c r="G434">
         <v>200</v>
@@ -13804,13 +13774,13 @@
         <v>9</v>
       </c>
       <c r="D435" t="s">
-        <v>570</v>
+        <v>584</v>
       </c>
       <c r="E435" t="s">
-        <v>232</v>
+        <v>585</v>
       </c>
       <c r="F435" t="s">
-        <v>232</v>
+        <v>585</v>
       </c>
       <c r="G435">
         <v>200</v>
@@ -13830,13 +13800,13 @@
         <v>9</v>
       </c>
       <c r="D436" t="s">
-        <v>571</v>
+        <v>586</v>
       </c>
       <c r="E436" t="s">
-        <v>572</v>
+        <v>42</v>
       </c>
       <c r="F436" t="s">
-        <v>572</v>
+        <v>42</v>
       </c>
       <c r="G436">
         <v>200</v>
@@ -13856,13 +13826,13 @@
         <v>9</v>
       </c>
       <c r="D437" t="s">
-        <v>573</v>
+        <v>587</v>
       </c>
       <c r="E437" t="s">
-        <v>312</v>
+        <v>270</v>
       </c>
       <c r="F437" t="s">
-        <v>312</v>
+        <v>270</v>
       </c>
       <c r="G437">
         <v>200</v>
@@ -13882,13 +13852,13 @@
         <v>9</v>
       </c>
       <c r="D438" t="s">
-        <v>574</v>
+        <v>588</v>
       </c>
       <c r="E438" t="s">
-        <v>304</v>
+        <v>262</v>
       </c>
       <c r="F438" t="s">
-        <v>304</v>
+        <v>262</v>
       </c>
       <c r="G438">
         <v>200</v>
@@ -13908,13 +13878,13 @@
         <v>9</v>
       </c>
       <c r="D439" t="s">
-        <v>575</v>
+        <v>589</v>
       </c>
       <c r="E439" t="s">
-        <v>323</v>
+        <v>590</v>
       </c>
       <c r="F439" t="s">
-        <v>323</v>
+        <v>590</v>
       </c>
       <c r="G439">
         <v>200</v>
@@ -13934,13 +13904,13 @@
         <v>9</v>
       </c>
       <c r="D440" t="s">
-        <v>576</v>
+        <v>591</v>
       </c>
       <c r="E440" t="s">
-        <v>361</v>
+        <v>592</v>
       </c>
       <c r="F440" t="s">
-        <v>361</v>
+        <v>592</v>
       </c>
       <c r="G440">
         <v>200</v>
@@ -13960,13 +13930,13 @@
         <v>9</v>
       </c>
       <c r="D441" t="s">
-        <v>577</v>
+        <v>593</v>
       </c>
       <c r="E441" t="s">
-        <v>296</v>
+        <v>594</v>
       </c>
       <c r="F441" t="s">
-        <v>296</v>
+        <v>594</v>
       </c>
       <c r="G441">
         <v>200</v>
@@ -13986,13 +13956,13 @@
         <v>9</v>
       </c>
       <c r="D442" t="s">
-        <v>578</v>
+        <v>595</v>
       </c>
       <c r="E442" t="s">
-        <v>374</v>
+        <v>596</v>
       </c>
       <c r="F442" t="s">
-        <v>374</v>
+        <v>596</v>
       </c>
       <c r="G442">
         <v>200</v>
@@ -14012,13 +13982,13 @@
         <v>9</v>
       </c>
       <c r="D443" t="s">
-        <v>579</v>
+        <v>597</v>
       </c>
       <c r="E443" t="s">
-        <v>153</v>
+        <v>52</v>
       </c>
       <c r="F443" t="s">
-        <v>153</v>
+        <v>52</v>
       </c>
       <c r="G443">
         <v>200</v>
@@ -14038,13 +14008,13 @@
         <v>9</v>
       </c>
       <c r="D444" t="s">
-        <v>580</v>
+        <v>598</v>
       </c>
       <c r="E444" t="s">
-        <v>372</v>
+        <v>599</v>
       </c>
       <c r="F444" t="s">
-        <v>372</v>
+        <v>599</v>
       </c>
       <c r="G444">
         <v>200</v>
@@ -14064,13 +14034,13 @@
         <v>9</v>
       </c>
       <c r="D445" t="s">
-        <v>581</v>
+        <v>600</v>
       </c>
       <c r="E445" t="s">
-        <v>368</v>
+        <v>601</v>
       </c>
       <c r="F445" t="s">
-        <v>368</v>
+        <v>601</v>
       </c>
       <c r="G445">
         <v>200</v>
@@ -14090,13 +14060,13 @@
         <v>9</v>
       </c>
       <c r="D446" t="s">
-        <v>582</v>
+        <v>602</v>
       </c>
       <c r="E446" t="s">
-        <v>387</v>
+        <v>603</v>
       </c>
       <c r="F446" t="s">
-        <v>387</v>
+        <v>603</v>
       </c>
       <c r="G446">
         <v>200</v>
@@ -14116,13 +14086,13 @@
         <v>9</v>
       </c>
       <c r="D447" t="s">
-        <v>583</v>
+        <v>604</v>
       </c>
       <c r="E447" t="s">
-        <v>193</v>
+        <v>605</v>
       </c>
       <c r="F447" t="s">
-        <v>193</v>
+        <v>605</v>
       </c>
       <c r="G447">
         <v>200</v>
@@ -14142,13 +14112,13 @@
         <v>9</v>
       </c>
       <c r="D448" t="s">
-        <v>584</v>
+        <v>606</v>
       </c>
       <c r="E448" t="s">
-        <v>385</v>
+        <v>607</v>
       </c>
       <c r="F448" t="s">
-        <v>385</v>
+        <v>607</v>
       </c>
       <c r="G448">
         <v>200</v>
@@ -14168,13 +14138,13 @@
         <v>9</v>
       </c>
       <c r="D449" t="s">
-        <v>585</v>
+        <v>608</v>
       </c>
       <c r="E449" t="s">
-        <v>382</v>
+        <v>609</v>
       </c>
       <c r="F449" t="s">
-        <v>382</v>
+        <v>609</v>
       </c>
       <c r="G449">
         <v>200</v>
@@ -14194,13 +14164,13 @@
         <v>9</v>
       </c>
       <c r="D450" t="s">
-        <v>586</v>
+        <v>610</v>
       </c>
       <c r="E450" t="s">
-        <v>587</v>
+        <v>114</v>
       </c>
       <c r="F450" t="s">
-        <v>587</v>
+        <v>114</v>
       </c>
       <c r="G450">
         <v>200</v>
@@ -14220,13 +14190,13 @@
         <v>9</v>
       </c>
       <c r="D451" t="s">
-        <v>588</v>
+        <v>176</v>
       </c>
       <c r="E451" t="s">
-        <v>391</v>
+        <v>177</v>
       </c>
       <c r="F451" t="s">
-        <v>391</v>
+        <v>177</v>
       </c>
       <c r="G451">
         <v>200</v>
@@ -14246,13 +14216,13 @@
         <v>9</v>
       </c>
       <c r="D452" t="s">
-        <v>589</v>
+        <v>611</v>
       </c>
       <c r="E452" t="s">
-        <v>590</v>
+        <v>283</v>
       </c>
       <c r="F452" t="s">
-        <v>590</v>
+        <v>283</v>
       </c>
       <c r="G452">
         <v>200</v>
@@ -14272,13 +14242,13 @@
         <v>9</v>
       </c>
       <c r="D453" t="s">
-        <v>591</v>
+        <v>612</v>
       </c>
       <c r="E453" t="s">
-        <v>592</v>
+        <v>613</v>
       </c>
       <c r="F453" t="s">
-        <v>592</v>
+        <v>613</v>
       </c>
       <c r="G453">
         <v>200</v>
@@ -14298,13 +14268,13 @@
         <v>9</v>
       </c>
       <c r="D454" t="s">
-        <v>593</v>
+        <v>614</v>
       </c>
       <c r="E454" t="s">
-        <v>395</v>
+        <v>48</v>
       </c>
       <c r="F454" t="s">
-        <v>395</v>
+        <v>48</v>
       </c>
       <c r="G454">
         <v>200</v>
@@ -14324,13 +14294,13 @@
         <v>9</v>
       </c>
       <c r="D455" t="s">
-        <v>594</v>
+        <v>19</v>
       </c>
       <c r="E455" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="F455" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="G455">
         <v>200</v>
@@ -14350,13 +14320,13 @@
         <v>9</v>
       </c>
       <c r="D456" t="s">
-        <v>595</v>
+        <v>615</v>
       </c>
       <c r="E456" t="s">
-        <v>429</v>
+        <v>616</v>
       </c>
       <c r="F456" t="s">
-        <v>429</v>
+        <v>616</v>
       </c>
       <c r="G456">
         <v>200</v>
@@ -14376,13 +14346,13 @@
         <v>9</v>
       </c>
       <c r="D457" t="s">
-        <v>596</v>
+        <v>617</v>
       </c>
       <c r="E457" t="s">
-        <v>597</v>
+        <v>618</v>
       </c>
       <c r="F457" t="s">
-        <v>597</v>
+        <v>618</v>
       </c>
       <c r="G457">
         <v>200</v>
@@ -14402,13 +14372,13 @@
         <v>9</v>
       </c>
       <c r="D458" t="s">
-        <v>598</v>
+        <v>619</v>
       </c>
       <c r="E458" t="s">
-        <v>42</v>
+        <v>620</v>
       </c>
       <c r="F458" t="s">
-        <v>42</v>
+        <v>620</v>
       </c>
       <c r="G458">
         <v>200</v>
@@ -14428,13 +14398,13 @@
         <v>9</v>
       </c>
       <c r="D459" t="s">
-        <v>599</v>
+        <v>621</v>
       </c>
       <c r="E459" t="s">
-        <v>270</v>
+        <v>618</v>
       </c>
       <c r="F459" t="s">
-        <v>270</v>
+        <v>618</v>
       </c>
       <c r="G459">
         <v>200</v>
@@ -14454,13 +14424,13 @@
         <v>9</v>
       </c>
       <c r="D460" t="s">
-        <v>600</v>
+        <v>622</v>
       </c>
       <c r="E460" t="s">
-        <v>262</v>
+        <v>620</v>
       </c>
       <c r="F460" t="s">
-        <v>262</v>
+        <v>620</v>
       </c>
       <c r="G460">
         <v>200</v>
@@ -14480,13 +14450,13 @@
         <v>9</v>
       </c>
       <c r="D461" t="s">
-        <v>601</v>
+        <v>23</v>
       </c>
       <c r="E461" t="s">
-        <v>602</v>
+        <v>24</v>
       </c>
       <c r="F461" t="s">
-        <v>602</v>
+        <v>24</v>
       </c>
       <c r="G461">
         <v>200</v>
@@ -14506,13 +14476,13 @@
         <v>9</v>
       </c>
       <c r="D462" t="s">
-        <v>603</v>
+        <v>623</v>
       </c>
       <c r="E462" t="s">
-        <v>604</v>
+        <v>624</v>
       </c>
       <c r="F462" t="s">
-        <v>604</v>
+        <v>624</v>
       </c>
       <c r="G462">
         <v>200</v>
@@ -14532,13 +14502,13 @@
         <v>9</v>
       </c>
       <c r="D463" t="s">
-        <v>605</v>
+        <v>625</v>
       </c>
       <c r="E463" t="s">
-        <v>545</v>
+        <v>22</v>
       </c>
       <c r="F463" t="s">
-        <v>545</v>
+        <v>22</v>
       </c>
       <c r="G463">
         <v>200</v>
@@ -14558,13 +14528,13 @@
         <v>9</v>
       </c>
       <c r="D464" t="s">
-        <v>606</v>
+        <v>626</v>
       </c>
       <c r="E464" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="F464" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="G464">
         <v>200</v>
@@ -14573,30 +14543,30 @@
         <v>11</v>
       </c>
     </row>
-    <row r="465" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A465">
+    <row r="465" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A465" s="5">
         <v>464</v>
       </c>
-      <c r="B465" t="s">
-        <v>8</v>
-      </c>
-      <c r="C465" t="s">
-        <v>9</v>
-      </c>
-      <c r="D465" t="s">
-        <v>608</v>
-      </c>
-      <c r="E465" t="s">
-        <v>52</v>
-      </c>
-      <c r="F465" t="s">
-        <v>52</v>
-      </c>
-      <c r="G465">
-        <v>200</v>
-      </c>
-      <c r="H465" s="2" t="s">
-        <v>11</v>
+      <c r="B465" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C465" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D465" s="5" t="s">
+        <v>628</v>
+      </c>
+      <c r="E465" s="5" t="s">
+        <v>629</v>
+      </c>
+      <c r="F465" s="5" t="s">
+        <v>629</v>
+      </c>
+      <c r="G465" s="6">
+        <v>400</v>
+      </c>
+      <c r="H465" s="6" t="s">
+        <v>630</v>
       </c>
     </row>
     <row r="466" spans="1:8" x14ac:dyDescent="0.25">
@@ -14610,13 +14580,13 @@
         <v>9</v>
       </c>
       <c r="D466" t="s">
-        <v>609</v>
+        <v>631</v>
       </c>
       <c r="E466" t="s">
-        <v>554</v>
+        <v>632</v>
       </c>
       <c r="F466" t="s">
-        <v>554</v>
+        <v>632</v>
       </c>
       <c r="G466">
         <v>200</v>
@@ -14636,13 +14606,13 @@
         <v>9</v>
       </c>
       <c r="D467" t="s">
-        <v>610</v>
+        <v>633</v>
       </c>
       <c r="E467" t="s">
-        <v>611</v>
+        <v>634</v>
       </c>
       <c r="F467" t="s">
-        <v>611</v>
+        <v>634</v>
       </c>
       <c r="G467">
         <v>200</v>
@@ -14662,13 +14632,13 @@
         <v>9</v>
       </c>
       <c r="D468" t="s">
-        <v>612</v>
+        <v>635</v>
       </c>
       <c r="E468" t="s">
-        <v>613</v>
+        <v>636</v>
       </c>
       <c r="F468" t="s">
-        <v>613</v>
+        <v>636</v>
       </c>
       <c r="G468">
         <v>200</v>
@@ -14688,13 +14658,13 @@
         <v>9</v>
       </c>
       <c r="D469" t="s">
-        <v>614</v>
+        <v>637</v>
       </c>
       <c r="E469" t="s">
-        <v>615</v>
+        <v>607</v>
       </c>
       <c r="F469" t="s">
-        <v>615</v>
+        <v>607</v>
       </c>
       <c r="G469">
         <v>200</v>
@@ -14714,13 +14684,13 @@
         <v>9</v>
       </c>
       <c r="D470" t="s">
-        <v>616</v>
+        <v>638</v>
       </c>
       <c r="E470" t="s">
-        <v>617</v>
+        <v>639</v>
       </c>
       <c r="F470" t="s">
-        <v>617</v>
+        <v>639</v>
       </c>
       <c r="G470">
         <v>200</v>
@@ -14740,13 +14710,13 @@
         <v>9</v>
       </c>
       <c r="D471" t="s">
-        <v>618</v>
+        <v>640</v>
       </c>
       <c r="E471" t="s">
-        <v>619</v>
+        <v>641</v>
       </c>
       <c r="F471" t="s">
-        <v>619</v>
+        <v>641</v>
       </c>
       <c r="G471">
         <v>200</v>
@@ -14766,13 +14736,13 @@
         <v>9</v>
       </c>
       <c r="D472" t="s">
-        <v>620</v>
+        <v>642</v>
       </c>
       <c r="E472" t="s">
-        <v>114</v>
+        <v>8</v>
       </c>
       <c r="F472" t="s">
-        <v>114</v>
+        <v>8</v>
       </c>
       <c r="G472">
         <v>200</v>
@@ -14792,13 +14762,13 @@
         <v>9</v>
       </c>
       <c r="D473" t="s">
-        <v>176</v>
+        <v>643</v>
       </c>
       <c r="E473" t="s">
-        <v>177</v>
+        <v>644</v>
       </c>
       <c r="F473" t="s">
-        <v>177</v>
+        <v>644</v>
       </c>
       <c r="G473">
         <v>200</v>
@@ -14818,13 +14788,13 @@
         <v>9</v>
       </c>
       <c r="D474" t="s">
-        <v>621</v>
+        <v>645</v>
       </c>
       <c r="E474" t="s">
-        <v>283</v>
+        <v>646</v>
       </c>
       <c r="F474" t="s">
-        <v>283</v>
+        <v>646</v>
       </c>
       <c r="G474">
         <v>200</v>
@@ -14844,13 +14814,13 @@
         <v>9</v>
       </c>
       <c r="D475" t="s">
-        <v>622</v>
+        <v>647</v>
       </c>
       <c r="E475" t="s">
-        <v>623</v>
+        <v>648</v>
       </c>
       <c r="F475" t="s">
-        <v>623</v>
+        <v>648</v>
       </c>
       <c r="G475">
         <v>200</v>
@@ -14870,13 +14840,13 @@
         <v>9</v>
       </c>
       <c r="D476" t="s">
-        <v>624</v>
+        <v>649</v>
       </c>
       <c r="E476" t="s">
-        <v>48</v>
+        <v>650</v>
       </c>
       <c r="F476" t="s">
-        <v>48</v>
+        <v>650</v>
       </c>
       <c r="G476">
         <v>200</v>
@@ -14896,13 +14866,13 @@
         <v>9</v>
       </c>
       <c r="D477" t="s">
-        <v>19</v>
+        <v>651</v>
       </c>
       <c r="E477" t="s">
-        <v>20</v>
+        <v>652</v>
       </c>
       <c r="F477" t="s">
-        <v>20</v>
+        <v>652</v>
       </c>
       <c r="G477">
         <v>200</v>
@@ -14922,13 +14892,13 @@
         <v>9</v>
       </c>
       <c r="D478" t="s">
-        <v>625</v>
+        <v>653</v>
       </c>
       <c r="E478" t="s">
-        <v>626</v>
+        <v>114</v>
       </c>
       <c r="F478" t="s">
-        <v>626</v>
+        <v>114</v>
       </c>
       <c r="G478">
         <v>200</v>
@@ -14948,13 +14918,13 @@
         <v>9</v>
       </c>
       <c r="D479" t="s">
-        <v>627</v>
+        <v>654</v>
       </c>
       <c r="E479" t="s">
-        <v>628</v>
+        <v>61</v>
       </c>
       <c r="F479" t="s">
-        <v>628</v>
+        <v>61</v>
       </c>
       <c r="G479">
         <v>200</v>
@@ -14974,13 +14944,13 @@
         <v>9</v>
       </c>
       <c r="D480" t="s">
-        <v>629</v>
+        <v>655</v>
       </c>
       <c r="E480" t="s">
-        <v>630</v>
+        <v>38</v>
       </c>
       <c r="F480" t="s">
-        <v>630</v>
+        <v>38</v>
       </c>
       <c r="G480">
         <v>200</v>
@@ -15000,13 +14970,13 @@
         <v>9</v>
       </c>
       <c r="D481" t="s">
-        <v>631</v>
+        <v>656</v>
       </c>
       <c r="E481" t="s">
-        <v>628</v>
+        <v>72</v>
       </c>
       <c r="F481" t="s">
-        <v>628</v>
+        <v>72</v>
       </c>
       <c r="G481">
         <v>200</v>
@@ -15026,13 +14996,13 @@
         <v>9</v>
       </c>
       <c r="D482" t="s">
-        <v>632</v>
+        <v>657</v>
       </c>
       <c r="E482" t="s">
-        <v>630</v>
+        <v>44</v>
       </c>
       <c r="F482" t="s">
-        <v>630</v>
+        <v>44</v>
       </c>
       <c r="G482">
         <v>200</v>
@@ -15052,13 +15022,13 @@
         <v>9</v>
       </c>
       <c r="D483" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="E483" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="F483" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="G483">
         <v>200</v>
@@ -15078,13 +15048,13 @@
         <v>9</v>
       </c>
       <c r="D484" t="s">
-        <v>633</v>
+        <v>658</v>
       </c>
       <c r="E484" t="s">
-        <v>634</v>
+        <v>149</v>
       </c>
       <c r="F484" t="s">
-        <v>634</v>
+        <v>149</v>
       </c>
       <c r="G484">
         <v>200</v>
@@ -15104,13 +15074,13 @@
         <v>9</v>
       </c>
       <c r="D485" t="s">
-        <v>635</v>
+        <v>659</v>
       </c>
       <c r="E485" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F485" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="G485">
         <v>200</v>
@@ -15130,13 +15100,13 @@
         <v>9</v>
       </c>
       <c r="D486" t="s">
-        <v>636</v>
+        <v>660</v>
       </c>
       <c r="E486" t="s">
-        <v>637</v>
+        <v>140</v>
       </c>
       <c r="F486" t="s">
-        <v>637</v>
+        <v>140</v>
       </c>
       <c r="G486">
         <v>200</v>
@@ -15145,30 +15115,30 @@
         <v>11</v>
       </c>
     </row>
-    <row r="487" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A487" s="5">
+    <row r="487" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A487">
         <v>486</v>
       </c>
-      <c r="B487" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C487" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D487" s="5" t="s">
-        <v>638</v>
-      </c>
-      <c r="E487" s="5" t="s">
-        <v>639</v>
-      </c>
-      <c r="F487" s="5" t="s">
-        <v>639</v>
-      </c>
-      <c r="G487" s="6">
-        <v>400</v>
-      </c>
-      <c r="H487" s="6" t="s">
-        <v>640</v>
+      <c r="B487" t="s">
+        <v>8</v>
+      </c>
+      <c r="C487" t="s">
+        <v>9</v>
+      </c>
+      <c r="D487" t="s">
+        <v>141</v>
+      </c>
+      <c r="E487" t="s">
+        <v>142</v>
+      </c>
+      <c r="F487" t="s">
+        <v>142</v>
+      </c>
+      <c r="G487">
+        <v>200</v>
+      </c>
+      <c r="H487" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="488" spans="1:8" x14ac:dyDescent="0.25">
@@ -15182,13 +15152,13 @@
         <v>9</v>
       </c>
       <c r="D488" t="s">
-        <v>641</v>
+        <v>371</v>
       </c>
       <c r="E488" t="s">
-        <v>642</v>
+        <v>372</v>
       </c>
       <c r="F488" t="s">
-        <v>642</v>
+        <v>372</v>
       </c>
       <c r="G488">
         <v>200</v>
@@ -15208,13 +15178,13 @@
         <v>9</v>
       </c>
       <c r="D489" t="s">
-        <v>643</v>
+        <v>116</v>
       </c>
       <c r="E489" t="s">
-        <v>644</v>
+        <v>98</v>
       </c>
       <c r="F489" t="s">
-        <v>644</v>
+        <v>98</v>
       </c>
       <c r="G489">
         <v>200</v>
@@ -15234,13 +15204,13 @@
         <v>9</v>
       </c>
       <c r="D490" t="s">
-        <v>645</v>
+        <v>39</v>
       </c>
       <c r="E490" t="s">
-        <v>646</v>
+        <v>40</v>
       </c>
       <c r="F490" t="s">
-        <v>646</v>
+        <v>40</v>
       </c>
       <c r="G490">
         <v>200</v>
@@ -15260,13 +15230,13 @@
         <v>9</v>
       </c>
       <c r="D491" t="s">
-        <v>647</v>
+        <v>661</v>
       </c>
       <c r="E491" t="s">
-        <v>617</v>
+        <v>290</v>
       </c>
       <c r="F491" t="s">
-        <v>617</v>
+        <v>290</v>
       </c>
       <c r="G491">
         <v>200</v>
@@ -15286,13 +15256,13 @@
         <v>9</v>
       </c>
       <c r="D492" t="s">
-        <v>648</v>
+        <v>662</v>
       </c>
       <c r="E492" t="s">
-        <v>649</v>
+        <v>288</v>
       </c>
       <c r="F492" t="s">
-        <v>649</v>
+        <v>288</v>
       </c>
       <c r="G492">
         <v>200</v>
@@ -15312,13 +15282,13 @@
         <v>9</v>
       </c>
       <c r="D493" t="s">
-        <v>650</v>
+        <v>663</v>
       </c>
       <c r="E493" t="s">
-        <v>651</v>
+        <v>157</v>
       </c>
       <c r="F493" t="s">
-        <v>651</v>
+        <v>157</v>
       </c>
       <c r="G493">
         <v>200</v>
@@ -15338,13 +15308,13 @@
         <v>9</v>
       </c>
       <c r="D494" t="s">
-        <v>652</v>
+        <v>178</v>
       </c>
       <c r="E494" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="F494" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="G494">
         <v>200</v>
@@ -15364,13 +15334,13 @@
         <v>9</v>
       </c>
       <c r="D495" t="s">
-        <v>653</v>
+        <v>200</v>
       </c>
       <c r="E495" t="s">
-        <v>654</v>
+        <v>201</v>
       </c>
       <c r="F495" t="s">
-        <v>654</v>
+        <v>201</v>
       </c>
       <c r="G495">
         <v>200</v>
@@ -15390,13 +15360,13 @@
         <v>9</v>
       </c>
       <c r="D496" t="s">
-        <v>655</v>
+        <v>196</v>
       </c>
       <c r="E496" t="s">
-        <v>656</v>
+        <v>197</v>
       </c>
       <c r="F496" t="s">
-        <v>656</v>
+        <v>197</v>
       </c>
       <c r="G496">
         <v>200</v>
@@ -15416,13 +15386,13 @@
         <v>9</v>
       </c>
       <c r="D497" t="s">
-        <v>657</v>
+        <v>198</v>
       </c>
       <c r="E497" t="s">
-        <v>658</v>
+        <v>199</v>
       </c>
       <c r="F497" t="s">
-        <v>658</v>
+        <v>199</v>
       </c>
       <c r="G497">
         <v>200</v>
@@ -15442,13 +15412,13 @@
         <v>9</v>
       </c>
       <c r="D498" t="s">
-        <v>659</v>
+        <v>664</v>
       </c>
       <c r="E498" t="s">
-        <v>660</v>
+        <v>28</v>
       </c>
       <c r="F498" t="s">
-        <v>660</v>
+        <v>28</v>
       </c>
       <c r="G498">
         <v>200</v>
@@ -15468,13 +15438,13 @@
         <v>9</v>
       </c>
       <c r="D499" t="s">
-        <v>661</v>
+        <v>224</v>
       </c>
       <c r="E499" t="s">
-        <v>662</v>
+        <v>223</v>
       </c>
       <c r="F499" t="s">
-        <v>662</v>
+        <v>223</v>
       </c>
       <c r="G499">
         <v>200</v>
@@ -15494,13 +15464,13 @@
         <v>9</v>
       </c>
       <c r="D500" t="s">
-        <v>663</v>
+        <v>225</v>
       </c>
       <c r="E500" t="s">
-        <v>114</v>
+        <v>226</v>
       </c>
       <c r="F500" t="s">
-        <v>114</v>
+        <v>226</v>
       </c>
       <c r="G500">
         <v>200</v>
@@ -15520,13 +15490,13 @@
         <v>9</v>
       </c>
       <c r="D501" t="s">
-        <v>664</v>
+        <v>204</v>
       </c>
       <c r="E501" t="s">
-        <v>61</v>
+        <v>205</v>
       </c>
       <c r="F501" t="s">
-        <v>61</v>
+        <v>205</v>
       </c>
       <c r="G501">
         <v>200</v>
@@ -15549,10 +15519,10 @@
         <v>665</v>
       </c>
       <c r="E502" t="s">
-        <v>38</v>
+        <v>155</v>
       </c>
       <c r="F502" t="s">
-        <v>38</v>
+        <v>155</v>
       </c>
       <c r="G502">
         <v>200</v>
@@ -15575,10 +15545,10 @@
         <v>666</v>
       </c>
       <c r="E503" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="F503" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="G503">
         <v>200</v>
@@ -15587,30 +15557,30 @@
         <v>11</v>
       </c>
     </row>
-    <row r="504" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A504">
+    <row r="504" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A504" s="3">
         <v>503</v>
       </c>
-      <c r="B504" t="s">
-        <v>8</v>
-      </c>
-      <c r="C504" t="s">
-        <v>9</v>
-      </c>
-      <c r="D504" t="s">
-        <v>667</v>
-      </c>
-      <c r="E504" t="s">
-        <v>44</v>
-      </c>
-      <c r="F504" t="s">
-        <v>44</v>
-      </c>
-      <c r="G504">
-        <v>200</v>
-      </c>
-      <c r="H504" s="2" t="s">
-        <v>11</v>
+      <c r="B504" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C504" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D504" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E504" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F504" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="G504" s="3">
+        <v>200</v>
+      </c>
+      <c r="H504" s="4" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="505" spans="1:8" x14ac:dyDescent="0.25">
@@ -15624,13 +15594,13 @@
         <v>9</v>
       </c>
       <c r="D505" t="s">
-        <v>41</v>
+        <v>667</v>
       </c>
       <c r="E505" t="s">
-        <v>42</v>
+        <v>122</v>
       </c>
       <c r="F505" t="s">
-        <v>42</v>
+        <v>122</v>
       </c>
       <c r="G505">
         <v>200</v>
@@ -15650,13 +15620,13 @@
         <v>9</v>
       </c>
       <c r="D506" t="s">
-        <v>668</v>
+        <v>322</v>
       </c>
       <c r="E506" t="s">
-        <v>149</v>
+        <v>323</v>
       </c>
       <c r="F506" t="s">
-        <v>149</v>
+        <v>323</v>
       </c>
       <c r="G506">
         <v>200</v>
@@ -15676,13 +15646,13 @@
         <v>9</v>
       </c>
       <c r="D507" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="E507" t="s">
-        <v>30</v>
+        <v>361</v>
       </c>
       <c r="F507" t="s">
-        <v>30</v>
+        <v>361</v>
       </c>
       <c r="G507">
         <v>200</v>
@@ -15702,13 +15672,13 @@
         <v>9</v>
       </c>
       <c r="D508" t="s">
-        <v>670</v>
+        <v>381</v>
       </c>
       <c r="E508" t="s">
-        <v>140</v>
+        <v>382</v>
       </c>
       <c r="F508" t="s">
-        <v>140</v>
+        <v>382</v>
       </c>
       <c r="G508">
         <v>200</v>
@@ -15728,13 +15698,13 @@
         <v>9</v>
       </c>
       <c r="D509" t="s">
-        <v>141</v>
+        <v>324</v>
       </c>
       <c r="E509" t="s">
-        <v>142</v>
+        <v>325</v>
       </c>
       <c r="F509" t="s">
-        <v>142</v>
+        <v>325</v>
       </c>
       <c r="G509">
         <v>200</v>
@@ -15754,13 +15724,13 @@
         <v>9</v>
       </c>
       <c r="D510" t="s">
-        <v>371</v>
+        <v>669</v>
       </c>
       <c r="E510" t="s">
-        <v>372</v>
+        <v>670</v>
       </c>
       <c r="F510" t="s">
-        <v>372</v>
+        <v>670</v>
       </c>
       <c r="G510">
         <v>200</v>
@@ -15780,13 +15750,13 @@
         <v>9</v>
       </c>
       <c r="D511" t="s">
-        <v>116</v>
+        <v>671</v>
       </c>
       <c r="E511" t="s">
-        <v>98</v>
+        <v>672</v>
       </c>
       <c r="F511" t="s">
-        <v>98</v>
+        <v>672</v>
       </c>
       <c r="G511">
         <v>200</v>
@@ -15806,13 +15776,13 @@
         <v>9</v>
       </c>
       <c r="D512" t="s">
-        <v>39</v>
+        <v>673</v>
       </c>
       <c r="E512" t="s">
-        <v>40</v>
+        <v>674</v>
       </c>
       <c r="F512" t="s">
-        <v>40</v>
+        <v>674</v>
       </c>
       <c r="G512">
         <v>200</v>
@@ -15832,13 +15802,13 @@
         <v>9</v>
       </c>
       <c r="D513" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="E513" t="s">
-        <v>290</v>
+        <v>676</v>
       </c>
       <c r="F513" t="s">
-        <v>290</v>
+        <v>676</v>
       </c>
       <c r="G513">
         <v>200</v>
@@ -15858,13 +15828,13 @@
         <v>9</v>
       </c>
       <c r="D514" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="E514" t="s">
-        <v>288</v>
+        <v>678</v>
       </c>
       <c r="F514" t="s">
-        <v>288</v>
+        <v>678</v>
       </c>
       <c r="G514">
         <v>200</v>
@@ -15884,13 +15854,13 @@
         <v>9</v>
       </c>
       <c r="D515" t="s">
-        <v>673</v>
+        <v>667</v>
       </c>
       <c r="E515" t="s">
-        <v>157</v>
+        <v>122</v>
       </c>
       <c r="F515" t="s">
-        <v>157</v>
+        <v>122</v>
       </c>
       <c r="G515">
         <v>200</v>
@@ -15910,13 +15880,13 @@
         <v>9</v>
       </c>
       <c r="D516" t="s">
-        <v>178</v>
+        <v>35</v>
       </c>
       <c r="E516" t="s">
-        <v>179</v>
+        <v>36</v>
       </c>
       <c r="F516" t="s">
-        <v>179</v>
+        <v>36</v>
       </c>
       <c r="G516">
         <v>200</v>
@@ -15936,13 +15906,13 @@
         <v>9</v>
       </c>
       <c r="D517" t="s">
-        <v>200</v>
+        <v>643</v>
       </c>
       <c r="E517" t="s">
-        <v>201</v>
+        <v>644</v>
       </c>
       <c r="F517" t="s">
-        <v>201</v>
+        <v>644</v>
       </c>
       <c r="G517">
         <v>200</v>
@@ -15962,590 +15932,18 @@
         <v>9</v>
       </c>
       <c r="D518" t="s">
-        <v>196</v>
+        <v>679</v>
       </c>
       <c r="E518" t="s">
-        <v>197</v>
+        <v>646</v>
       </c>
       <c r="F518" t="s">
-        <v>197</v>
+        <v>646</v>
       </c>
       <c r="G518">
         <v>200</v>
       </c>
       <c r="H518" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="519" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A519">
-        <v>518</v>
-      </c>
-      <c r="B519" t="s">
-        <v>8</v>
-      </c>
-      <c r="C519" t="s">
-        <v>9</v>
-      </c>
-      <c r="D519" t="s">
-        <v>198</v>
-      </c>
-      <c r="E519" t="s">
-        <v>199</v>
-      </c>
-      <c r="F519" t="s">
-        <v>199</v>
-      </c>
-      <c r="G519">
-        <v>200</v>
-      </c>
-      <c r="H519" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="520" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A520">
-        <v>519</v>
-      </c>
-      <c r="B520" t="s">
-        <v>8</v>
-      </c>
-      <c r="C520" t="s">
-        <v>9</v>
-      </c>
-      <c r="D520" t="s">
-        <v>674</v>
-      </c>
-      <c r="E520" t="s">
-        <v>28</v>
-      </c>
-      <c r="F520" t="s">
-        <v>28</v>
-      </c>
-      <c r="G520">
-        <v>200</v>
-      </c>
-      <c r="H520" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="521" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A521">
-        <v>520</v>
-      </c>
-      <c r="B521" t="s">
-        <v>8</v>
-      </c>
-      <c r="C521" t="s">
-        <v>9</v>
-      </c>
-      <c r="D521" t="s">
-        <v>224</v>
-      </c>
-      <c r="E521" t="s">
-        <v>223</v>
-      </c>
-      <c r="F521" t="s">
-        <v>223</v>
-      </c>
-      <c r="G521">
-        <v>200</v>
-      </c>
-      <c r="H521" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="522" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A522">
-        <v>521</v>
-      </c>
-      <c r="B522" t="s">
-        <v>8</v>
-      </c>
-      <c r="C522" t="s">
-        <v>9</v>
-      </c>
-      <c r="D522" t="s">
-        <v>225</v>
-      </c>
-      <c r="E522" t="s">
-        <v>226</v>
-      </c>
-      <c r="F522" t="s">
-        <v>226</v>
-      </c>
-      <c r="G522">
-        <v>200</v>
-      </c>
-      <c r="H522" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="523" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A523">
-        <v>522</v>
-      </c>
-      <c r="B523" t="s">
-        <v>8</v>
-      </c>
-      <c r="C523" t="s">
-        <v>9</v>
-      </c>
-      <c r="D523" t="s">
-        <v>204</v>
-      </c>
-      <c r="E523" t="s">
-        <v>205</v>
-      </c>
-      <c r="F523" t="s">
-        <v>205</v>
-      </c>
-      <c r="G523">
-        <v>200</v>
-      </c>
-      <c r="H523" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="524" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A524">
-        <v>523</v>
-      </c>
-      <c r="B524" t="s">
-        <v>8</v>
-      </c>
-      <c r="C524" t="s">
-        <v>9</v>
-      </c>
-      <c r="D524" t="s">
-        <v>675</v>
-      </c>
-      <c r="E524" t="s">
-        <v>155</v>
-      </c>
-      <c r="F524" t="s">
-        <v>155</v>
-      </c>
-      <c r="G524">
-        <v>200</v>
-      </c>
-      <c r="H524" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="525" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A525">
-        <v>524</v>
-      </c>
-      <c r="B525" t="s">
-        <v>8</v>
-      </c>
-      <c r="C525" t="s">
-        <v>9</v>
-      </c>
-      <c r="D525" t="s">
-        <v>676</v>
-      </c>
-      <c r="E525" t="s">
-        <v>80</v>
-      </c>
-      <c r="F525" t="s">
-        <v>80</v>
-      </c>
-      <c r="G525">
-        <v>200</v>
-      </c>
-      <c r="H525" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="526" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A526" s="3">
-        <v>525</v>
-      </c>
-      <c r="B526" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C526" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D526" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="E526" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="F526" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="G526" s="3">
-        <v>200</v>
-      </c>
-      <c r="H526" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="527" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A527">
-        <v>526</v>
-      </c>
-      <c r="B527" t="s">
-        <v>8</v>
-      </c>
-      <c r="C527" t="s">
-        <v>9</v>
-      </c>
-      <c r="D527" t="s">
-        <v>677</v>
-      </c>
-      <c r="E527" t="s">
-        <v>122</v>
-      </c>
-      <c r="F527" t="s">
-        <v>122</v>
-      </c>
-      <c r="G527">
-        <v>200</v>
-      </c>
-      <c r="H527" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="528" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A528">
-        <v>527</v>
-      </c>
-      <c r="B528" t="s">
-        <v>8</v>
-      </c>
-      <c r="C528" t="s">
-        <v>9</v>
-      </c>
-      <c r="D528" t="s">
-        <v>322</v>
-      </c>
-      <c r="E528" t="s">
-        <v>323</v>
-      </c>
-      <c r="F528" t="s">
-        <v>323</v>
-      </c>
-      <c r="G528">
-        <v>200</v>
-      </c>
-      <c r="H528" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="529" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A529">
-        <v>528</v>
-      </c>
-      <c r="B529" t="s">
-        <v>8</v>
-      </c>
-      <c r="C529" t="s">
-        <v>9</v>
-      </c>
-      <c r="D529" t="s">
-        <v>678</v>
-      </c>
-      <c r="E529" t="s">
-        <v>361</v>
-      </c>
-      <c r="F529" t="s">
-        <v>361</v>
-      </c>
-      <c r="G529">
-        <v>200</v>
-      </c>
-      <c r="H529" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="530" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A530">
-        <v>529</v>
-      </c>
-      <c r="B530" t="s">
-        <v>8</v>
-      </c>
-      <c r="C530" t="s">
-        <v>9</v>
-      </c>
-      <c r="D530" t="s">
-        <v>381</v>
-      </c>
-      <c r="E530" t="s">
-        <v>382</v>
-      </c>
-      <c r="F530" t="s">
-        <v>382</v>
-      </c>
-      <c r="G530">
-        <v>200</v>
-      </c>
-      <c r="H530" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="531" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A531">
-        <v>530</v>
-      </c>
-      <c r="B531" t="s">
-        <v>8</v>
-      </c>
-      <c r="C531" t="s">
-        <v>9</v>
-      </c>
-      <c r="D531" t="s">
-        <v>324</v>
-      </c>
-      <c r="E531" t="s">
-        <v>325</v>
-      </c>
-      <c r="F531" t="s">
-        <v>325</v>
-      </c>
-      <c r="G531">
-        <v>200</v>
-      </c>
-      <c r="H531" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="532" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A532">
-        <v>531</v>
-      </c>
-      <c r="B532" t="s">
-        <v>8</v>
-      </c>
-      <c r="C532" t="s">
-        <v>9</v>
-      </c>
-      <c r="D532" t="s">
-        <v>679</v>
-      </c>
-      <c r="E532" t="s">
-        <v>680</v>
-      </c>
-      <c r="F532" t="s">
-        <v>680</v>
-      </c>
-      <c r="G532">
-        <v>200</v>
-      </c>
-      <c r="H532" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="533" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A533">
-        <v>532</v>
-      </c>
-      <c r="B533" t="s">
-        <v>8</v>
-      </c>
-      <c r="C533" t="s">
-        <v>9</v>
-      </c>
-      <c r="D533" t="s">
-        <v>681</v>
-      </c>
-      <c r="E533" t="s">
-        <v>682</v>
-      </c>
-      <c r="F533" t="s">
-        <v>682</v>
-      </c>
-      <c r="G533">
-        <v>200</v>
-      </c>
-      <c r="H533" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="534" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A534">
-        <v>533</v>
-      </c>
-      <c r="B534" t="s">
-        <v>8</v>
-      </c>
-      <c r="C534" t="s">
-        <v>9</v>
-      </c>
-      <c r="D534" t="s">
-        <v>683</v>
-      </c>
-      <c r="E534" t="s">
-        <v>684</v>
-      </c>
-      <c r="F534" t="s">
-        <v>684</v>
-      </c>
-      <c r="G534">
-        <v>200</v>
-      </c>
-      <c r="H534" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="535" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A535">
-        <v>534</v>
-      </c>
-      <c r="B535" t="s">
-        <v>8</v>
-      </c>
-      <c r="C535" t="s">
-        <v>9</v>
-      </c>
-      <c r="D535" t="s">
-        <v>685</v>
-      </c>
-      <c r="E535" t="s">
-        <v>686</v>
-      </c>
-      <c r="F535" t="s">
-        <v>686</v>
-      </c>
-      <c r="G535">
-        <v>200</v>
-      </c>
-      <c r="H535" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="536" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A536">
-        <v>535</v>
-      </c>
-      <c r="B536" t="s">
-        <v>8</v>
-      </c>
-      <c r="C536" t="s">
-        <v>9</v>
-      </c>
-      <c r="D536" t="s">
-        <v>687</v>
-      </c>
-      <c r="E536" t="s">
-        <v>688</v>
-      </c>
-      <c r="F536" t="s">
-        <v>688</v>
-      </c>
-      <c r="G536">
-        <v>200</v>
-      </c>
-      <c r="H536" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="537" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A537">
-        <v>536</v>
-      </c>
-      <c r="B537" t="s">
-        <v>8</v>
-      </c>
-      <c r="C537" t="s">
-        <v>9</v>
-      </c>
-      <c r="D537" t="s">
-        <v>677</v>
-      </c>
-      <c r="E537" t="s">
-        <v>122</v>
-      </c>
-      <c r="F537" t="s">
-        <v>122</v>
-      </c>
-      <c r="G537">
-        <v>200</v>
-      </c>
-      <c r="H537" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="538" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A538">
-        <v>537</v>
-      </c>
-      <c r="B538" t="s">
-        <v>8</v>
-      </c>
-      <c r="C538" t="s">
-        <v>9</v>
-      </c>
-      <c r="D538" t="s">
-        <v>35</v>
-      </c>
-      <c r="E538" t="s">
-        <v>36</v>
-      </c>
-      <c r="F538" t="s">
-        <v>36</v>
-      </c>
-      <c r="G538">
-        <v>200</v>
-      </c>
-      <c r="H538" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="539" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A539">
-        <v>538</v>
-      </c>
-      <c r="B539" t="s">
-        <v>8</v>
-      </c>
-      <c r="C539" t="s">
-        <v>9</v>
-      </c>
-      <c r="D539" t="s">
-        <v>653</v>
-      </c>
-      <c r="E539" t="s">
-        <v>654</v>
-      </c>
-      <c r="F539" t="s">
-        <v>654</v>
-      </c>
-      <c r="G539">
-        <v>200</v>
-      </c>
-      <c r="H539" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="540" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A540">
-        <v>539</v>
-      </c>
-      <c r="B540" t="s">
-        <v>8</v>
-      </c>
-      <c r="C540" t="s">
-        <v>9</v>
-      </c>
-      <c r="D540" t="s">
-        <v>689</v>
-      </c>
-      <c r="E540" t="s">
-        <v>656</v>
-      </c>
-      <c r="F540" t="s">
-        <v>656</v>
-      </c>
-      <c r="G540">
-        <v>200</v>
-      </c>
-      <c r="H540" s="2" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Re-audit all 404 links on new Beta homepage
</commit_message>
<xml_diff>
--- a/Homepage_Links_Navigation_Report.xlsx
+++ b/Homepage_Links_Navigation_Report.xlsx
@@ -1609,6 +1609,12 @@
     <t>Wooden Street Sofa</t>
   </si>
   <si>
+    <t>woodenstreet - All Sofa cum bed</t>
+  </si>
+  <si>
+    <t>woodenstreet - All Coffee &amp; Centre Table</t>
+  </si>
+  <si>
     <t>woodenstreet - TV Units</t>
   </si>
   <si>
@@ -1622,12 +1628,6 @@
   </si>
   <si>
     <t>woodenstreet - All Study Tables</t>
-  </si>
-  <si>
-    <t>woodenstreet - All Sofa cum bed</t>
-  </si>
-  <si>
-    <t>woodenstreet - All Coffee &amp; Centre Table</t>
   </si>
   <si>
     <t>PULL UP A CHAIR</t>
@@ -12373,10 +12373,10 @@
         <v>532</v>
       </c>
       <c r="E381" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="F381" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="G381">
         <v>200</v>
@@ -12399,10 +12399,10 @@
         <v>533</v>
       </c>
       <c r="E382" t="s">
-        <v>385</v>
+        <v>504</v>
       </c>
       <c r="F382" t="s">
-        <v>385</v>
+        <v>504</v>
       </c>
       <c r="G382">
         <v>200</v>
@@ -12425,10 +12425,10 @@
         <v>534</v>
       </c>
       <c r="E383" t="s">
-        <v>535</v>
+        <v>44</v>
       </c>
       <c r="F383" t="s">
-        <v>535</v>
+        <v>44</v>
       </c>
       <c r="G383">
         <v>200</v>
@@ -12448,13 +12448,13 @@
         <v>9</v>
       </c>
       <c r="D384" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="E384" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
       <c r="F384" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
       <c r="G384">
         <v>200</v>
@@ -12474,13 +12474,13 @@
         <v>9</v>
       </c>
       <c r="D385" t="s">
+        <v>536</v>
+      </c>
+      <c r="E385" t="s">
         <v>537</v>
       </c>
-      <c r="E385" t="s">
-        <v>70</v>
-      </c>
       <c r="F385" t="s">
-        <v>70</v>
+        <v>537</v>
       </c>
       <c r="G385">
         <v>200</v>
@@ -12503,10 +12503,10 @@
         <v>538</v>
       </c>
       <c r="E386" t="s">
-        <v>504</v>
+        <v>370</v>
       </c>
       <c r="F386" t="s">
-        <v>504</v>
+        <v>370</v>
       </c>
       <c r="G386">
         <v>200</v>

</xml_diff>

<commit_message>
feat: Add Live homepage links, navigation & redirection audit report and dashboard for Desktop and Mobile
</commit_message>
<xml_diff>
--- a/Homepage_Links_Navigation_Report.xlsx
+++ b/Homepage_Links_Navigation_Report.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="All Links Audit" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Redirection Audit" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4559" uniqueCount="738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4611" uniqueCount="745">
   <si>
     <t>ID</t>
   </si>
@@ -1950,46 +1951,42 @@
 [2m    - accept-encoding: gzip,deflate,br[22m
 [2m    - Accept-Language: en-US,en;q=0.9[22m
 [2m    - Cache-Control: no-cache[22m
-[2m  - ← 301 Apple WebObjects 5.9.8-1[22m
-[2m    - connection: keep-alive[22m
-[2m    - content-length: 0[22m
+[2m  - ← 301 Moved Permanently[22m
 [2m    - server: daiquiri/5[22m
 [2m    - content-type: text/html; charset=UTF-8[22m
-[2m    - x-apple-jingle-correlation-key: 4VDH7XVLVKLAPPVPVRKEBOTA4Y[22m
-[2m    - x-apple-request-uuid: e5467fde-abaa-9607-beaf-ac5440ba60e6[22m
+[2m    - content-length: 0[22m
+[2m    - x-apple-jingle-correlation-key: MV6NIZWYLEBAMZY43E4NS22Q5E[22m
+[2m    - x-apple-request-uuid: 657cd466-d859-0206-671c-d938d96b50e9[22m
 [2m    - x-apple-translated-wo-url: /WebObjects/MZStore.woa/wa/viewSoftware?ls=1&amp;id=1162068644&amp;cc=in&amp;urlDesc=/wooden-street[22m
 [2m    - apple-tk: false[22m
-[2m    - x-b3-spanid: 420a6ab8538940ef[22m
-[2m    - edge-control: cache-maxage=0s, cache-maxage=0s[22m
+[2m    - x-b3-spanid: f09acc21e855d5fa[22m
 [2m    - x-apple-lokamai-no-cache: true, true[22m
-[2m    - b3: e5467fdeabaa9607beafac5440ba60e6-420a6ab8538940ef[22m
+[2m    - b3: 657cd466d8590206671cd938d96b50e9-f09acc21e855d5fa[22m
 [2m    - cache-control: max-age=0, max-age=0, no-store[22m
-[2m    - x-apple-aka-ttl: Generated Mon Sep 28 05:28:11 PDT 2026, Expires Mon Sep 28 05:28:11 PDT 2026, TTL 0s, cache-maxage=0s[22m
-[2m    - x-b3-traceid: e5467fdeabaa9607beafac5440ba60e6[22m
+[2m    - x-apple-aka-ttl: Generated Mon Sep 28 05:53:01 PDT 2026, Expires Mon Sep 28 05:53:01 PDT 2026, TTL 0s, cache-maxage=0s[22m
+[2m    - x-b3-traceid: 657cd466d8590206671cd938d96b50e9[22m
 [2m    - x-webobjects-loadaverage: 0[22m
-[2m    - last-modified: Mon, 28 Sep 2026 12:28:11 GMT[22m
+[2m    - last-modified: Mon, 28 Sep 2026 12:53:01 GMT[22m
 [2m    - apple-seq: 0.0[22m
 [2m    - access-control-allow-origin: *[22m
 [2m    - apple-originating-system: MZStore[22m
 [2m    - strict-transport-security: max-age=31536000; includeSubDomains[22m
 [2m    - x-frame-options: SAMEORIGIN[22m
 [2m    - x-apple-orig-url: https://apps.apple.com/in/app/wooden-street/id1162068644?ls=1[22m
-[2m    - x-apple-application-site: ST11[22m
+[2m    - x-apple-application-site: MR22[22m
 [2m    - apple-timing-app: 3 ms[22m
 [2m    - location: itms-appss://apps.apple.com/in/app/wooden-street/id1162068644?ls=1[22m
-[2m    - x-apple-application-instance: 2500196[22m
-[2m    - x-responding-instance: MZStore:2500196:::[22m
-[2m    - x-daiquiri-instance: daiquiri:41896014:st47p00it-qujn12071501:7987:26RELEASE153:daiquiri-amp-store-l7shared-int-001-st, daiquiri:41896001:st53p00it-qujn12040301:7987:26RELEASE153:daiquiri-amp-store-l7shared-int-001-st, daiquiri:42282007:st53p00it-qujn11032102:7987:26RELEASE153:daiquiri-amp-store-l7shared-ext-001-st[22m
-[2m    - x-daiquiri-debug-worker-pid: 75044, 2310, 102174[22m
-[2m    - accept-ranges: bytes[22m
-[2m    - date: Mon, 28 Sep 2026 12:28:11 GMT[22m
-[2m    - via: 1.1 varnish[22m
-[2m    - x-cdn: fsly[22m
-[2m    - x-served-by: cache-maa10220-MAA[22m
-[2m    - x-cache-hits: 0[22m
-[2m    - x-timer: S1790598491.467521,VS0,VE294[22m
-[2m    - set-cookie: geo=IN; domain=apple.com[22m
-[2m    - x-cache: MISS fsly[22m
+[2m    - x-apple-application-instance: 3500163[22m
+[2m    - x-responding-instance: MZStore:3500163:::[22m
+[2m    - x-daiquiri-instance: daiquiri:11896010:mr50p00it-qujn12072902:7987:26RELEASE153:daiquiri-amp-store-l7shared-int-001-mr, daiquiri:11896007:mr47p00it-qujn04123002:7987:26RELEASE153:daiquiri-amp-store-l7shared-int-001-mr, daiquiri:12282001:mr47p00it-qujn06080702:7987:26RELEASE153:daiquiri-amp-store-l7shared-ext-001-mr[22m
+[2m    - x-daiquiri-debug-worker-pid: 34030, 43099, 108974[22m
+[2m    - date: Mon, 28 Sep 2026 12:53:01 GMT[22m
+[2m    - x-cache: TCP_REFRESH_MISS from a23-48-245-229.deploy.akamaitechnologies.com (AkamaiGHost/22.6.4-888a2d21768272d5e2d80e9762941e76) (S)[22m
+[2m    - connection: keep-alive[22m
+[2m    - x-cache-remote: TCP_REFRESH_MISS from a184-86-112-215.deploy.akamaitechnologies.com (AkamaiGHost/22.6.3-da071da6976b6d633b0b37bcfe65c0fc) (S)[22m
+[2m    - set-cookie: geo=IN; domain=.apple.com[22m
+[2m    - alt-svc: h3=":443"; ma=93600[22m
+[2m    - vary: X-Apple-Store-Front, Cookie[22m
 )</t>
   </si>
   <si>
@@ -2254,6 +2251,24 @@
     <t>Wooden Street</t>
   </si>
   <si>
+    <t>View Product</t>
+  </si>
+  <si>
+    <t>https://www.woodenstreet.com/product/feltro-sofa-cum-bed-honey-finish</t>
+  </si>
+  <si>
+    <t>https://www.woodenstreet.com/product/lorenz-3-seater-sofa-cotton-jade-ivory</t>
+  </si>
+  <si>
+    <t>https://www.woodenstreet.com/product/waver-4-seater-outdoor-dining-set</t>
+  </si>
+  <si>
+    <t>https://www.woodenstreet.com/product/walken-bed-with-storage-honey-finish</t>
+  </si>
+  <si>
+    <t>View All</t>
+  </si>
+  <si>
     <t>Get it on Google Play</t>
   </si>
   <si>
@@ -2273,6 +2288,9 @@
   </si>
   <si>
     <t>Certification - Verification of Compliance of BIFMA</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
@@ -2305,7 +2323,7 @@
       <color rgb="991B1B"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2327,6 +2345,11 @@
         <fgColor rgb="FEE2E2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="D97706"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -2340,7 +2363,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2350,6 +2373,9 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2689,7 +2715,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H759"/>
+  <dimension ref="A1:H764"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -16351,56 +16377,56 @@
         <v>12</v>
       </c>
     </row>
-    <row r="526" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A526" s="3">
+    <row r="526" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A526">
         <v>525</v>
       </c>
-      <c r="B526" s="3" t="s">
-        <v>682</v>
-      </c>
-      <c r="C526" s="3" t="s">
+      <c r="B526" t="s">
+        <v>682</v>
+      </c>
+      <c r="C526" t="s">
         <v>685</v>
       </c>
-      <c r="D526" s="3" t="s">
+      <c r="D526" t="s">
         <v>691</v>
       </c>
-      <c r="E526" s="3" t="s">
+      <c r="E526" t="s">
         <v>692</v>
       </c>
-      <c r="F526" s="3" t="s">
+      <c r="F526" t="s">
         <v>693</v>
       </c>
-      <c r="G526" s="3">
-        <v>200</v>
-      </c>
-      <c r="H526" s="4" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="527" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A527" s="3">
+      <c r="G526">
+        <v>200</v>
+      </c>
+      <c r="H526" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="527" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A527">
         <v>526</v>
       </c>
-      <c r="B527" s="3" t="s">
-        <v>682</v>
-      </c>
-      <c r="C527" s="3" t="s">
+      <c r="B527" t="s">
+        <v>682</v>
+      </c>
+      <c r="C527" t="s">
         <v>685</v>
       </c>
-      <c r="D527" s="3" t="s">
+      <c r="D527" t="s">
         <v>694</v>
       </c>
-      <c r="E527" s="3" t="s">
+      <c r="E527" t="s">
         <v>695</v>
       </c>
-      <c r="F527" s="3" t="s">
+      <c r="F527" t="s">
         <v>597</v>
       </c>
-      <c r="G527" s="3">
-        <v>200</v>
-      </c>
-      <c r="H527" s="4" t="s">
-        <v>137</v>
+      <c r="G527">
+        <v>200</v>
+      </c>
+      <c r="H527" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="528" spans="1:8" x14ac:dyDescent="0.25">
@@ -19456,13 +19482,13 @@
         <v>697</v>
       </c>
       <c r="D645" t="s">
-        <v>544</v>
+        <v>731</v>
       </c>
       <c r="E645" t="s">
-        <v>545</v>
+        <v>732</v>
       </c>
       <c r="F645" t="s">
-        <v>545</v>
+        <v>732</v>
       </c>
       <c r="G645">
         <v>200</v>
@@ -19482,13 +19508,13 @@
         <v>697</v>
       </c>
       <c r="D646" t="s">
-        <v>546</v>
+        <v>731</v>
       </c>
       <c r="E646" t="s">
-        <v>62</v>
+        <v>733</v>
       </c>
       <c r="F646" t="s">
-        <v>62</v>
+        <v>733</v>
       </c>
       <c r="G646">
         <v>200</v>
@@ -19508,13 +19534,13 @@
         <v>697</v>
       </c>
       <c r="D647" t="s">
-        <v>547</v>
+        <v>731</v>
       </c>
       <c r="E647" t="s">
-        <v>89</v>
+        <v>734</v>
       </c>
       <c r="F647" t="s">
-        <v>89</v>
+        <v>734</v>
       </c>
       <c r="G647">
         <v>200</v>
@@ -19534,13 +19560,13 @@
         <v>697</v>
       </c>
       <c r="D648" t="s">
-        <v>548</v>
+        <v>731</v>
       </c>
       <c r="E648" t="s">
-        <v>31</v>
+        <v>735</v>
       </c>
       <c r="F648" t="s">
-        <v>31</v>
+        <v>735</v>
       </c>
       <c r="G648">
         <v>200</v>
@@ -19560,13 +19586,13 @@
         <v>697</v>
       </c>
       <c r="D649" t="s">
-        <v>549</v>
+        <v>736</v>
       </c>
       <c r="E649" t="s">
-        <v>172</v>
+        <v>600</v>
       </c>
       <c r="F649" t="s">
-        <v>172</v>
+        <v>600</v>
       </c>
       <c r="G649">
         <v>200</v>
@@ -19586,13 +19612,13 @@
         <v>697</v>
       </c>
       <c r="D650" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="E650" t="s">
-        <v>45</v>
+        <v>545</v>
       </c>
       <c r="F650" t="s">
-        <v>45</v>
+        <v>545</v>
       </c>
       <c r="G650">
         <v>200</v>
@@ -19612,13 +19638,13 @@
         <v>697</v>
       </c>
       <c r="D651" t="s">
-        <v>82</v>
+        <v>546</v>
       </c>
       <c r="E651" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="F651" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="G651">
         <v>200</v>
@@ -19638,13 +19664,13 @@
         <v>697</v>
       </c>
       <c r="D652" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
       <c r="E652" t="s">
-        <v>202</v>
+        <v>89</v>
       </c>
       <c r="F652" t="s">
-        <v>202</v>
+        <v>89</v>
       </c>
       <c r="G652">
         <v>200</v>
@@ -19664,13 +19690,13 @@
         <v>697</v>
       </c>
       <c r="D653" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="E653" t="s">
-        <v>200</v>
+        <v>31</v>
       </c>
       <c r="F653" t="s">
-        <v>200</v>
+        <v>31</v>
       </c>
       <c r="G653">
         <v>200</v>
@@ -19690,13 +19716,13 @@
         <v>697</v>
       </c>
       <c r="D654" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="E654" t="s">
-        <v>81</v>
+        <v>172</v>
       </c>
       <c r="F654" t="s">
-        <v>81</v>
+        <v>172</v>
       </c>
       <c r="G654">
         <v>200</v>
@@ -19716,13 +19742,13 @@
         <v>697</v>
       </c>
       <c r="D655" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="E655" t="s">
-        <v>227</v>
+        <v>45</v>
       </c>
       <c r="F655" t="s">
-        <v>227</v>
+        <v>45</v>
       </c>
       <c r="G655">
         <v>200</v>
@@ -19742,13 +19768,13 @@
         <v>697</v>
       </c>
       <c r="D656" t="s">
-        <v>555</v>
+        <v>82</v>
       </c>
       <c r="E656" t="s">
-        <v>556</v>
+        <v>33</v>
       </c>
       <c r="F656" t="s">
-        <v>556</v>
+        <v>33</v>
       </c>
       <c r="G656">
         <v>200</v>
@@ -19768,13 +19794,13 @@
         <v>697</v>
       </c>
       <c r="D657" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="E657" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="F657" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="G657">
         <v>200</v>
@@ -19794,13 +19820,13 @@
         <v>697</v>
       </c>
       <c r="D658" t="s">
-        <v>558</v>
+        <v>552</v>
       </c>
       <c r="E658" t="s">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="F658" t="s">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="G658">
         <v>200</v>
@@ -19820,13 +19846,13 @@
         <v>697</v>
       </c>
       <c r="D659" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="E659" t="s">
-        <v>233</v>
+        <v>81</v>
       </c>
       <c r="F659" t="s">
-        <v>233</v>
+        <v>81</v>
       </c>
       <c r="G659">
         <v>200</v>
@@ -19846,13 +19872,13 @@
         <v>697</v>
       </c>
       <c r="D660" t="s">
-        <v>560</v>
+        <v>554</v>
       </c>
       <c r="E660" t="s">
-        <v>561</v>
+        <v>227</v>
       </c>
       <c r="F660" t="s">
-        <v>561</v>
+        <v>227</v>
       </c>
       <c r="G660">
         <v>200</v>
@@ -19872,13 +19898,13 @@
         <v>697</v>
       </c>
       <c r="D661" t="s">
-        <v>562</v>
+        <v>555</v>
       </c>
       <c r="E661" t="s">
-        <v>313</v>
+        <v>556</v>
       </c>
       <c r="F661" t="s">
-        <v>313</v>
+        <v>556</v>
       </c>
       <c r="G661">
         <v>200</v>
@@ -19898,13 +19924,13 @@
         <v>697</v>
       </c>
       <c r="D662" t="s">
-        <v>563</v>
+        <v>557</v>
       </c>
       <c r="E662" t="s">
-        <v>305</v>
+        <v>206</v>
       </c>
       <c r="F662" t="s">
-        <v>305</v>
+        <v>206</v>
       </c>
       <c r="G662">
         <v>200</v>
@@ -19924,13 +19950,13 @@
         <v>697</v>
       </c>
       <c r="D663" t="s">
-        <v>564</v>
+        <v>558</v>
       </c>
       <c r="E663" t="s">
-        <v>324</v>
+        <v>180</v>
       </c>
       <c r="F663" t="s">
-        <v>324</v>
+        <v>180</v>
       </c>
       <c r="G663">
         <v>200</v>
@@ -19950,13 +19976,13 @@
         <v>697</v>
       </c>
       <c r="D664" t="s">
-        <v>565</v>
+        <v>559</v>
       </c>
       <c r="E664" t="s">
-        <v>362</v>
+        <v>233</v>
       </c>
       <c r="F664" t="s">
-        <v>362</v>
+        <v>233</v>
       </c>
       <c r="G664">
         <v>200</v>
@@ -19976,13 +20002,13 @@
         <v>697</v>
       </c>
       <c r="D665" t="s">
-        <v>566</v>
+        <v>560</v>
       </c>
       <c r="E665" t="s">
-        <v>297</v>
+        <v>561</v>
       </c>
       <c r="F665" t="s">
-        <v>297</v>
+        <v>561</v>
       </c>
       <c r="G665">
         <v>200</v>
@@ -20002,13 +20028,13 @@
         <v>697</v>
       </c>
       <c r="D666" t="s">
-        <v>567</v>
+        <v>562</v>
       </c>
       <c r="E666" t="s">
-        <v>375</v>
+        <v>313</v>
       </c>
       <c r="F666" t="s">
-        <v>375</v>
+        <v>313</v>
       </c>
       <c r="G666">
         <v>200</v>
@@ -20028,13 +20054,13 @@
         <v>697</v>
       </c>
       <c r="D667" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="E667" t="s">
-        <v>154</v>
+        <v>305</v>
       </c>
       <c r="F667" t="s">
-        <v>154</v>
+        <v>305</v>
       </c>
       <c r="G667">
         <v>200</v>
@@ -20054,13 +20080,13 @@
         <v>697</v>
       </c>
       <c r="D668" t="s">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="E668" t="s">
-        <v>373</v>
+        <v>324</v>
       </c>
       <c r="F668" t="s">
-        <v>373</v>
+        <v>324</v>
       </c>
       <c r="G668">
         <v>200</v>
@@ -20080,13 +20106,13 @@
         <v>697</v>
       </c>
       <c r="D669" t="s">
-        <v>570</v>
+        <v>565</v>
       </c>
       <c r="E669" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="F669" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="G669">
         <v>200</v>
@@ -20106,13 +20132,13 @@
         <v>697</v>
       </c>
       <c r="D670" t="s">
-        <v>571</v>
+        <v>566</v>
       </c>
       <c r="E670" t="s">
-        <v>388</v>
+        <v>297</v>
       </c>
       <c r="F670" t="s">
-        <v>388</v>
+        <v>297</v>
       </c>
       <c r="G670">
         <v>200</v>
@@ -20132,13 +20158,13 @@
         <v>697</v>
       </c>
       <c r="D671" t="s">
-        <v>572</v>
+        <v>567</v>
       </c>
       <c r="E671" t="s">
-        <v>194</v>
+        <v>375</v>
       </c>
       <c r="F671" t="s">
-        <v>194</v>
+        <v>375</v>
       </c>
       <c r="G671">
         <v>200</v>
@@ -20158,13 +20184,13 @@
         <v>697</v>
       </c>
       <c r="D672" t="s">
-        <v>573</v>
+        <v>568</v>
       </c>
       <c r="E672" t="s">
-        <v>386</v>
+        <v>154</v>
       </c>
       <c r="F672" t="s">
-        <v>386</v>
+        <v>154</v>
       </c>
       <c r="G672">
         <v>200</v>
@@ -20184,13 +20210,13 @@
         <v>697</v>
       </c>
       <c r="D673" t="s">
-        <v>574</v>
+        <v>569</v>
       </c>
       <c r="E673" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
       <c r="F673" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
       <c r="G673">
         <v>200</v>
@@ -20210,13 +20236,13 @@
         <v>697</v>
       </c>
       <c r="D674" t="s">
-        <v>575</v>
+        <v>570</v>
       </c>
       <c r="E674" t="s">
-        <v>576</v>
+        <v>369</v>
       </c>
       <c r="F674" t="s">
-        <v>576</v>
+        <v>369</v>
       </c>
       <c r="G674">
         <v>200</v>
@@ -20236,13 +20262,13 @@
         <v>697</v>
       </c>
       <c r="D675" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
       <c r="E675" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="F675" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="G675">
         <v>200</v>
@@ -20262,13 +20288,13 @@
         <v>697</v>
       </c>
       <c r="D676" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="E676" t="s">
-        <v>579</v>
+        <v>194</v>
       </c>
       <c r="F676" t="s">
-        <v>579</v>
+        <v>194</v>
       </c>
       <c r="G676">
         <v>200</v>
@@ -20288,13 +20314,13 @@
         <v>697</v>
       </c>
       <c r="D677" t="s">
-        <v>580</v>
+        <v>573</v>
       </c>
       <c r="E677" t="s">
-        <v>581</v>
+        <v>386</v>
       </c>
       <c r="F677" t="s">
-        <v>581</v>
+        <v>386</v>
       </c>
       <c r="G677">
         <v>200</v>
@@ -20314,13 +20340,13 @@
         <v>697</v>
       </c>
       <c r="D678" t="s">
-        <v>582</v>
+        <v>574</v>
       </c>
       <c r="E678" t="s">
-        <v>396</v>
+        <v>383</v>
       </c>
       <c r="F678" t="s">
-        <v>396</v>
+        <v>383</v>
       </c>
       <c r="G678">
         <v>200</v>
@@ -20340,13 +20366,13 @@
         <v>697</v>
       </c>
       <c r="D679" t="s">
-        <v>583</v>
+        <v>575</v>
       </c>
       <c r="E679" t="s">
-        <v>47</v>
+        <v>576</v>
       </c>
       <c r="F679" t="s">
-        <v>47</v>
+        <v>576</v>
       </c>
       <c r="G679">
         <v>200</v>
@@ -20366,13 +20392,13 @@
         <v>697</v>
       </c>
       <c r="D680" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="E680" t="s">
-        <v>430</v>
+        <v>392</v>
       </c>
       <c r="F680" t="s">
-        <v>430</v>
+        <v>392</v>
       </c>
       <c r="G680">
         <v>200</v>
@@ -20392,13 +20418,13 @@
         <v>697</v>
       </c>
       <c r="D681" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="E681" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="F681" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="G681">
         <v>200</v>
@@ -20418,13 +20444,13 @@
         <v>697</v>
       </c>
       <c r="D682" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
       <c r="E682" t="s">
-        <v>43</v>
+        <v>581</v>
       </c>
       <c r="F682" t="s">
-        <v>43</v>
+        <v>581</v>
       </c>
       <c r="G682">
         <v>200</v>
@@ -20444,13 +20470,13 @@
         <v>697</v>
       </c>
       <c r="D683" t="s">
-        <v>588</v>
+        <v>582</v>
       </c>
       <c r="E683" t="s">
-        <v>271</v>
+        <v>396</v>
       </c>
       <c r="F683" t="s">
-        <v>271</v>
+        <v>396</v>
       </c>
       <c r="G683">
         <v>200</v>
@@ -20470,13 +20496,13 @@
         <v>697</v>
       </c>
       <c r="D684" t="s">
-        <v>589</v>
+        <v>583</v>
       </c>
       <c r="E684" t="s">
-        <v>263</v>
+        <v>47</v>
       </c>
       <c r="F684" t="s">
-        <v>263</v>
+        <v>47</v>
       </c>
       <c r="G684">
         <v>200</v>
@@ -20496,13 +20522,13 @@
         <v>697</v>
       </c>
       <c r="D685" t="s">
-        <v>731</v>
+        <v>584</v>
       </c>
       <c r="E685" t="s">
-        <v>639</v>
+        <v>430</v>
       </c>
       <c r="F685" t="s">
-        <v>639</v>
+        <v>430</v>
       </c>
       <c r="G685">
         <v>200</v>
@@ -20511,30 +20537,30 @@
         <v>12</v>
       </c>
     </row>
-    <row r="686" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A686" s="5">
+    <row r="686" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A686">
         <v>685</v>
       </c>
-      <c r="B686" s="5" t="s">
-        <v>682</v>
-      </c>
-      <c r="C686" s="5" t="s">
-        <v>697</v>
-      </c>
-      <c r="D686" s="5" t="s">
-        <v>732</v>
-      </c>
-      <c r="E686" s="5" t="s">
-        <v>641</v>
-      </c>
-      <c r="F686" s="5" t="s">
-        <v>641</v>
-      </c>
-      <c r="G686" s="6" t="s">
-        <v>642</v>
-      </c>
-      <c r="H686" s="6" t="s">
-        <v>643</v>
+      <c r="B686" t="s">
+        <v>682</v>
+      </c>
+      <c r="C686" t="s">
+        <v>697</v>
+      </c>
+      <c r="D686" t="s">
+        <v>585</v>
+      </c>
+      <c r="E686" t="s">
+        <v>586</v>
+      </c>
+      <c r="F686" t="s">
+        <v>586</v>
+      </c>
+      <c r="G686">
+        <v>200</v>
+      </c>
+      <c r="H686" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="687" spans="1:8" x14ac:dyDescent="0.25">
@@ -20548,13 +20574,13 @@
         <v>697</v>
       </c>
       <c r="D687" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="E687" t="s">
-        <v>591</v>
+        <v>43</v>
       </c>
       <c r="F687" t="s">
-        <v>591</v>
+        <v>43</v>
       </c>
       <c r="G687">
         <v>200</v>
@@ -20574,13 +20600,13 @@
         <v>697</v>
       </c>
       <c r="D688" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E688" t="s">
-        <v>593</v>
+        <v>271</v>
       </c>
       <c r="F688" t="s">
-        <v>593</v>
+        <v>271</v>
       </c>
       <c r="G688">
         <v>200</v>
@@ -20600,13 +20626,13 @@
         <v>697</v>
       </c>
       <c r="D689" t="s">
-        <v>594</v>
+        <v>589</v>
       </c>
       <c r="E689" t="s">
-        <v>595</v>
+        <v>263</v>
       </c>
       <c r="F689" t="s">
-        <v>595</v>
+        <v>263</v>
       </c>
       <c r="G689">
         <v>200</v>
@@ -20626,13 +20652,13 @@
         <v>697</v>
       </c>
       <c r="D690" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="E690" t="s">
-        <v>625</v>
+        <v>639</v>
       </c>
       <c r="F690" t="s">
-        <v>625</v>
+        <v>639</v>
       </c>
       <c r="G690">
         <v>200</v>
@@ -20641,30 +20667,30 @@
         <v>12</v>
       </c>
     </row>
-    <row r="691" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A691">
+    <row r="691" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A691" s="5">
         <v>690</v>
       </c>
-      <c r="B691" t="s">
-        <v>682</v>
-      </c>
-      <c r="C691" t="s">
-        <v>697</v>
-      </c>
-      <c r="D691" t="s">
-        <v>599</v>
-      </c>
-      <c r="E691" t="s">
-        <v>600</v>
-      </c>
-      <c r="F691" t="s">
-        <v>600</v>
-      </c>
-      <c r="G691">
-        <v>200</v>
-      </c>
-      <c r="H691" s="2" t="s">
-        <v>12</v>
+      <c r="B691" s="5" t="s">
+        <v>682</v>
+      </c>
+      <c r="C691" s="5" t="s">
+        <v>697</v>
+      </c>
+      <c r="D691" s="5" t="s">
+        <v>738</v>
+      </c>
+      <c r="E691" s="5" t="s">
+        <v>641</v>
+      </c>
+      <c r="F691" s="5" t="s">
+        <v>641</v>
+      </c>
+      <c r="G691" s="6" t="s">
+        <v>642</v>
+      </c>
+      <c r="H691" s="6" t="s">
+        <v>643</v>
       </c>
     </row>
     <row r="692" spans="1:8" x14ac:dyDescent="0.25">
@@ -20678,13 +20704,13 @@
         <v>697</v>
       </c>
       <c r="D692" t="s">
-        <v>601</v>
+        <v>590</v>
       </c>
       <c r="E692" t="s">
-        <v>602</v>
+        <v>591</v>
       </c>
       <c r="F692" t="s">
-        <v>602</v>
+        <v>591</v>
       </c>
       <c r="G692">
         <v>200</v>
@@ -20704,13 +20730,13 @@
         <v>697</v>
       </c>
       <c r="D693" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="E693" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="F693" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="G693">
         <v>200</v>
@@ -20730,13 +20756,13 @@
         <v>697</v>
       </c>
       <c r="D694" t="s">
-        <v>611</v>
+        <v>594</v>
       </c>
       <c r="E694" t="s">
-        <v>115</v>
+        <v>595</v>
       </c>
       <c r="F694" t="s">
-        <v>115</v>
+        <v>595</v>
       </c>
       <c r="G694">
         <v>200</v>
@@ -20756,13 +20782,13 @@
         <v>697</v>
       </c>
       <c r="D695" t="s">
-        <v>177</v>
+        <v>739</v>
       </c>
       <c r="E695" t="s">
-        <v>178</v>
+        <v>625</v>
       </c>
       <c r="F695" t="s">
-        <v>178</v>
+        <v>625</v>
       </c>
       <c r="G695">
         <v>200</v>
@@ -20782,13 +20808,13 @@
         <v>697</v>
       </c>
       <c r="D696" t="s">
-        <v>612</v>
+        <v>599</v>
       </c>
       <c r="E696" t="s">
-        <v>284</v>
+        <v>600</v>
       </c>
       <c r="F696" t="s">
-        <v>284</v>
+        <v>600</v>
       </c>
       <c r="G696">
         <v>200</v>
@@ -20808,13 +20834,13 @@
         <v>697</v>
       </c>
       <c r="D697" t="s">
-        <v>347</v>
+        <v>601</v>
       </c>
       <c r="E697" t="s">
-        <v>152</v>
+        <v>602</v>
       </c>
       <c r="F697" t="s">
-        <v>152</v>
+        <v>602</v>
       </c>
       <c r="G697">
         <v>200</v>
@@ -20834,13 +20860,13 @@
         <v>697</v>
       </c>
       <c r="D698" t="s">
-        <v>400</v>
+        <v>596</v>
       </c>
       <c r="E698" t="s">
-        <v>401</v>
+        <v>597</v>
       </c>
       <c r="F698" t="s">
-        <v>401</v>
+        <v>597</v>
       </c>
       <c r="G698">
         <v>200</v>
@@ -20860,13 +20886,13 @@
         <v>697</v>
       </c>
       <c r="D699" t="s">
-        <v>46</v>
+        <v>611</v>
       </c>
       <c r="E699" t="s">
-        <v>47</v>
+        <v>115</v>
       </c>
       <c r="F699" t="s">
-        <v>47</v>
+        <v>115</v>
       </c>
       <c r="G699">
         <v>200</v>
@@ -20886,13 +20912,13 @@
         <v>697</v>
       </c>
       <c r="D700" t="s">
-        <v>598</v>
+        <v>177</v>
       </c>
       <c r="E700" t="s">
-        <v>53</v>
+        <v>178</v>
       </c>
       <c r="F700" t="s">
-        <v>53</v>
+        <v>178</v>
       </c>
       <c r="G700">
         <v>200</v>
@@ -20912,13 +20938,13 @@
         <v>697</v>
       </c>
       <c r="D701" t="s">
-        <v>603</v>
+        <v>612</v>
       </c>
       <c r="E701" t="s">
-        <v>604</v>
+        <v>284</v>
       </c>
       <c r="F701" t="s">
-        <v>604</v>
+        <v>284</v>
       </c>
       <c r="G701">
         <v>200</v>
@@ -20938,13 +20964,13 @@
         <v>697</v>
       </c>
       <c r="D702" t="s">
-        <v>609</v>
+        <v>347</v>
       </c>
       <c r="E702" t="s">
-        <v>610</v>
+        <v>152</v>
       </c>
       <c r="F702" t="s">
-        <v>610</v>
+        <v>152</v>
       </c>
       <c r="G702">
         <v>200</v>
@@ -20964,13 +20990,13 @@
         <v>697</v>
       </c>
       <c r="D703" t="s">
-        <v>616</v>
+        <v>400</v>
       </c>
       <c r="E703" t="s">
-        <v>617</v>
+        <v>401</v>
       </c>
       <c r="F703" t="s">
-        <v>617</v>
+        <v>401</v>
       </c>
       <c r="G703">
         <v>200</v>
@@ -20990,13 +21016,13 @@
         <v>697</v>
       </c>
       <c r="D704" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="E704" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="F704" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="G704">
         <v>200</v>
@@ -21016,13 +21042,13 @@
         <v>697</v>
       </c>
       <c r="D705" t="s">
-        <v>734</v>
+        <v>598</v>
       </c>
       <c r="E705" t="s">
-        <v>735</v>
+        <v>53</v>
       </c>
       <c r="F705" t="s">
-        <v>735</v>
+        <v>53</v>
       </c>
       <c r="G705">
         <v>200</v>
@@ -21042,13 +21068,13 @@
         <v>697</v>
       </c>
       <c r="D706" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="E706" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="F706" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="G706">
         <v>200</v>
@@ -21068,13 +21094,13 @@
         <v>697</v>
       </c>
       <c r="D707" t="s">
-        <v>15</v>
+        <v>609</v>
       </c>
       <c r="E707" t="s">
-        <v>16</v>
+        <v>610</v>
       </c>
       <c r="F707" t="s">
-        <v>16</v>
+        <v>610</v>
       </c>
       <c r="G707">
         <v>200</v>
@@ -21094,13 +21120,13 @@
         <v>697</v>
       </c>
       <c r="D708" t="s">
-        <v>645</v>
+        <v>616</v>
       </c>
       <c r="E708" t="s">
-        <v>646</v>
+        <v>617</v>
       </c>
       <c r="F708" t="s">
-        <v>646</v>
+        <v>617</v>
       </c>
       <c r="G708">
         <v>200</v>
@@ -21120,13 +21146,13 @@
         <v>697</v>
       </c>
       <c r="D709" t="s">
-        <v>647</v>
+        <v>20</v>
       </c>
       <c r="E709" t="s">
-        <v>648</v>
+        <v>21</v>
       </c>
       <c r="F709" t="s">
-        <v>648</v>
+        <v>21</v>
       </c>
       <c r="G709">
         <v>200</v>
@@ -21146,13 +21172,13 @@
         <v>697</v>
       </c>
       <c r="D710" t="s">
-        <v>649</v>
+        <v>740</v>
       </c>
       <c r="E710" t="s">
-        <v>650</v>
+        <v>741</v>
       </c>
       <c r="F710" t="s">
-        <v>650</v>
+        <v>741</v>
       </c>
       <c r="G710">
         <v>200</v>
@@ -21172,13 +21198,13 @@
         <v>697</v>
       </c>
       <c r="D711" t="s">
-        <v>651</v>
+        <v>605</v>
       </c>
       <c r="E711" t="s">
-        <v>652</v>
+        <v>606</v>
       </c>
       <c r="F711" t="s">
-        <v>652</v>
+        <v>606</v>
       </c>
       <c r="G711">
         <v>200</v>
@@ -21198,13 +21224,13 @@
         <v>697</v>
       </c>
       <c r="D712" t="s">
-        <v>653</v>
+        <v>15</v>
       </c>
       <c r="E712" t="s">
-        <v>654</v>
+        <v>16</v>
       </c>
       <c r="F712" t="s">
-        <v>654</v>
+        <v>16</v>
       </c>
       <c r="G712">
         <v>200</v>
@@ -21224,13 +21250,13 @@
         <v>697</v>
       </c>
       <c r="D713" t="s">
-        <v>736</v>
+        <v>645</v>
       </c>
       <c r="E713" t="s">
-        <v>619</v>
+        <v>646</v>
       </c>
       <c r="F713" t="s">
-        <v>619</v>
+        <v>646</v>
       </c>
       <c r="G713">
         <v>200</v>
@@ -21250,13 +21276,13 @@
         <v>697</v>
       </c>
       <c r="D714" t="s">
-        <v>737</v>
+        <v>647</v>
       </c>
       <c r="E714" t="s">
-        <v>621</v>
+        <v>648</v>
       </c>
       <c r="F714" t="s">
-        <v>621</v>
+        <v>648</v>
       </c>
       <c r="G714">
         <v>200</v>
@@ -21276,13 +21302,13 @@
         <v>697</v>
       </c>
       <c r="D715" t="s">
-        <v>627</v>
+        <v>649</v>
       </c>
       <c r="E715" t="s">
-        <v>628</v>
+        <v>650</v>
       </c>
       <c r="F715" t="s">
-        <v>628</v>
+        <v>650</v>
       </c>
       <c r="G715">
         <v>200</v>
@@ -21302,13 +21328,13 @@
         <v>697</v>
       </c>
       <c r="D716" t="s">
-        <v>629</v>
+        <v>651</v>
       </c>
       <c r="E716" t="s">
-        <v>630</v>
+        <v>652</v>
       </c>
       <c r="F716" t="s">
-        <v>630</v>
+        <v>652</v>
       </c>
       <c r="G716">
         <v>200</v>
@@ -21328,13 +21354,13 @@
         <v>697</v>
       </c>
       <c r="D717" t="s">
-        <v>631</v>
+        <v>653</v>
       </c>
       <c r="E717" t="s">
-        <v>632</v>
+        <v>654</v>
       </c>
       <c r="F717" t="s">
-        <v>632</v>
+        <v>654</v>
       </c>
       <c r="G717">
         <v>200</v>
@@ -21354,13 +21380,13 @@
         <v>697</v>
       </c>
       <c r="D718" t="s">
-        <v>633</v>
+        <v>742</v>
       </c>
       <c r="E718" t="s">
-        <v>634</v>
+        <v>619</v>
       </c>
       <c r="F718" t="s">
-        <v>634</v>
+        <v>619</v>
       </c>
       <c r="G718">
         <v>200</v>
@@ -21380,13 +21406,13 @@
         <v>697</v>
       </c>
       <c r="D719" t="s">
-        <v>635</v>
+        <v>743</v>
       </c>
       <c r="E719" t="s">
-        <v>636</v>
+        <v>621</v>
       </c>
       <c r="F719" t="s">
-        <v>636</v>
+        <v>621</v>
       </c>
       <c r="G719">
         <v>200</v>
@@ -21406,13 +21432,13 @@
         <v>697</v>
       </c>
       <c r="D720" t="s">
-        <v>655</v>
+        <v>627</v>
       </c>
       <c r="E720" t="s">
-        <v>115</v>
+        <v>628</v>
       </c>
       <c r="F720" t="s">
-        <v>115</v>
+        <v>628</v>
       </c>
       <c r="G720">
         <v>200</v>
@@ -21432,13 +21458,13 @@
         <v>697</v>
       </c>
       <c r="D721" t="s">
-        <v>656</v>
+        <v>629</v>
       </c>
       <c r="E721" t="s">
-        <v>62</v>
+        <v>630</v>
       </c>
       <c r="F721" t="s">
-        <v>62</v>
+        <v>630</v>
       </c>
       <c r="G721">
         <v>200</v>
@@ -21458,13 +21484,13 @@
         <v>697</v>
       </c>
       <c r="D722" t="s">
-        <v>657</v>
+        <v>631</v>
       </c>
       <c r="E722" t="s">
-        <v>39</v>
+        <v>632</v>
       </c>
       <c r="F722" t="s">
-        <v>39</v>
+        <v>632</v>
       </c>
       <c r="G722">
         <v>200</v>
@@ -21484,13 +21510,13 @@
         <v>697</v>
       </c>
       <c r="D723" t="s">
-        <v>658</v>
+        <v>633</v>
       </c>
       <c r="E723" t="s">
-        <v>73</v>
+        <v>634</v>
       </c>
       <c r="F723" t="s">
-        <v>73</v>
+        <v>634</v>
       </c>
       <c r="G723">
         <v>200</v>
@@ -21510,13 +21536,13 @@
         <v>697</v>
       </c>
       <c r="D724" t="s">
-        <v>659</v>
+        <v>635</v>
       </c>
       <c r="E724" t="s">
-        <v>45</v>
+        <v>636</v>
       </c>
       <c r="F724" t="s">
-        <v>45</v>
+        <v>636</v>
       </c>
       <c r="G724">
         <v>200</v>
@@ -21536,13 +21562,13 @@
         <v>697</v>
       </c>
       <c r="D725" t="s">
-        <v>42</v>
+        <v>655</v>
       </c>
       <c r="E725" t="s">
-        <v>43</v>
+        <v>115</v>
       </c>
       <c r="F725" t="s">
-        <v>43</v>
+        <v>115</v>
       </c>
       <c r="G725">
         <v>200</v>
@@ -21562,13 +21588,13 @@
         <v>697</v>
       </c>
       <c r="D726" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="E726" t="s">
-        <v>150</v>
+        <v>62</v>
       </c>
       <c r="F726" t="s">
-        <v>150</v>
+        <v>62</v>
       </c>
       <c r="G726">
         <v>200</v>
@@ -21588,13 +21614,13 @@
         <v>697</v>
       </c>
       <c r="D727" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="E727" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="F727" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="G727">
         <v>200</v>
@@ -21614,13 +21640,13 @@
         <v>697</v>
       </c>
       <c r="D728" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="E728" t="s">
-        <v>141</v>
+        <v>73</v>
       </c>
       <c r="F728" t="s">
-        <v>141</v>
+        <v>73</v>
       </c>
       <c r="G728">
         <v>200</v>
@@ -21640,13 +21666,13 @@
         <v>697</v>
       </c>
       <c r="D729" t="s">
-        <v>142</v>
+        <v>659</v>
       </c>
       <c r="E729" t="s">
-        <v>143</v>
+        <v>45</v>
       </c>
       <c r="F729" t="s">
-        <v>143</v>
+        <v>45</v>
       </c>
       <c r="G729">
         <v>200</v>
@@ -21666,13 +21692,13 @@
         <v>697</v>
       </c>
       <c r="D730" t="s">
-        <v>372</v>
+        <v>42</v>
       </c>
       <c r="E730" t="s">
-        <v>373</v>
+        <v>43</v>
       </c>
       <c r="F730" t="s">
-        <v>373</v>
+        <v>43</v>
       </c>
       <c r="G730">
         <v>200</v>
@@ -21692,13 +21718,13 @@
         <v>697</v>
       </c>
       <c r="D731" t="s">
-        <v>117</v>
+        <v>660</v>
       </c>
       <c r="E731" t="s">
-        <v>99</v>
+        <v>150</v>
       </c>
       <c r="F731" t="s">
-        <v>99</v>
+        <v>150</v>
       </c>
       <c r="G731">
         <v>200</v>
@@ -21718,13 +21744,13 @@
         <v>697</v>
       </c>
       <c r="D732" t="s">
-        <v>40</v>
+        <v>661</v>
       </c>
       <c r="E732" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F732" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="G732">
         <v>200</v>
@@ -21744,13 +21770,13 @@
         <v>697</v>
       </c>
       <c r="D733" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E733" t="s">
-        <v>291</v>
+        <v>141</v>
       </c>
       <c r="F733" t="s">
-        <v>291</v>
+        <v>141</v>
       </c>
       <c r="G733">
         <v>200</v>
@@ -21770,13 +21796,13 @@
         <v>697</v>
       </c>
       <c r="D734" t="s">
-        <v>664</v>
+        <v>142</v>
       </c>
       <c r="E734" t="s">
-        <v>289</v>
+        <v>143</v>
       </c>
       <c r="F734" t="s">
-        <v>289</v>
+        <v>143</v>
       </c>
       <c r="G734">
         <v>200</v>
@@ -21796,13 +21822,13 @@
         <v>697</v>
       </c>
       <c r="D735" t="s">
-        <v>665</v>
+        <v>372</v>
       </c>
       <c r="E735" t="s">
-        <v>158</v>
+        <v>373</v>
       </c>
       <c r="F735" t="s">
-        <v>158</v>
+        <v>373</v>
       </c>
       <c r="G735">
         <v>200</v>
@@ -21822,13 +21848,13 @@
         <v>697</v>
       </c>
       <c r="D736" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
       <c r="E736" t="s">
-        <v>180</v>
+        <v>99</v>
       </c>
       <c r="F736" t="s">
-        <v>180</v>
+        <v>99</v>
       </c>
       <c r="G736">
         <v>200</v>
@@ -21848,13 +21874,13 @@
         <v>697</v>
       </c>
       <c r="D737" t="s">
-        <v>201</v>
+        <v>40</v>
       </c>
       <c r="E737" t="s">
-        <v>202</v>
+        <v>41</v>
       </c>
       <c r="F737" t="s">
-        <v>202</v>
+        <v>41</v>
       </c>
       <c r="G737">
         <v>200</v>
@@ -21874,13 +21900,13 @@
         <v>697</v>
       </c>
       <c r="D738" t="s">
-        <v>197</v>
+        <v>663</v>
       </c>
       <c r="E738" t="s">
-        <v>198</v>
+        <v>291</v>
       </c>
       <c r="F738" t="s">
-        <v>198</v>
+        <v>291</v>
       </c>
       <c r="G738">
         <v>200</v>
@@ -21900,13 +21926,13 @@
         <v>697</v>
       </c>
       <c r="D739" t="s">
-        <v>199</v>
+        <v>664</v>
       </c>
       <c r="E739" t="s">
-        <v>200</v>
+        <v>289</v>
       </c>
       <c r="F739" t="s">
-        <v>200</v>
+        <v>289</v>
       </c>
       <c r="G739">
         <v>200</v>
@@ -21926,13 +21952,13 @@
         <v>697</v>
       </c>
       <c r="D740" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="E740" t="s">
-        <v>29</v>
+        <v>158</v>
       </c>
       <c r="F740" t="s">
-        <v>29</v>
+        <v>158</v>
       </c>
       <c r="G740">
         <v>200</v>
@@ -21952,13 +21978,13 @@
         <v>697</v>
       </c>
       <c r="D741" t="s">
-        <v>225</v>
+        <v>179</v>
       </c>
       <c r="E741" t="s">
-        <v>224</v>
+        <v>180</v>
       </c>
       <c r="F741" t="s">
-        <v>224</v>
+        <v>180</v>
       </c>
       <c r="G741">
         <v>200</v>
@@ -21978,13 +22004,13 @@
         <v>697</v>
       </c>
       <c r="D742" t="s">
-        <v>226</v>
+        <v>201</v>
       </c>
       <c r="E742" t="s">
-        <v>227</v>
+        <v>202</v>
       </c>
       <c r="F742" t="s">
-        <v>227</v>
+        <v>202</v>
       </c>
       <c r="G742">
         <v>200</v>
@@ -22004,13 +22030,13 @@
         <v>697</v>
       </c>
       <c r="D743" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="E743" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="F743" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="G743">
         <v>200</v>
@@ -22030,13 +22056,13 @@
         <v>697</v>
       </c>
       <c r="D744" t="s">
-        <v>667</v>
+        <v>199</v>
       </c>
       <c r="E744" t="s">
-        <v>156</v>
+        <v>200</v>
       </c>
       <c r="F744" t="s">
-        <v>156</v>
+        <v>200</v>
       </c>
       <c r="G744">
         <v>200</v>
@@ -22056,13 +22082,13 @@
         <v>697</v>
       </c>
       <c r="D745" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="E745" t="s">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="F745" t="s">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="G745">
         <v>200</v>
@@ -22071,30 +22097,30 @@
         <v>12</v>
       </c>
     </row>
-    <row r="746" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A746" s="3">
+    <row r="746" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A746">
         <v>745</v>
       </c>
-      <c r="B746" s="3" t="s">
-        <v>682</v>
-      </c>
-      <c r="C746" s="3" t="s">
-        <v>697</v>
-      </c>
-      <c r="D746" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E746" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="F746" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="G746" s="3">
-        <v>200</v>
-      </c>
-      <c r="H746" s="4" t="s">
-        <v>137</v>
+      <c r="B746" t="s">
+        <v>682</v>
+      </c>
+      <c r="C746" t="s">
+        <v>697</v>
+      </c>
+      <c r="D746" t="s">
+        <v>225</v>
+      </c>
+      <c r="E746" t="s">
+        <v>224</v>
+      </c>
+      <c r="F746" t="s">
+        <v>224</v>
+      </c>
+      <c r="G746">
+        <v>200</v>
+      </c>
+      <c r="H746" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="747" spans="1:8" x14ac:dyDescent="0.25">
@@ -22108,13 +22134,13 @@
         <v>697</v>
       </c>
       <c r="D747" t="s">
-        <v>669</v>
+        <v>226</v>
       </c>
       <c r="E747" t="s">
-        <v>123</v>
+        <v>227</v>
       </c>
       <c r="F747" t="s">
-        <v>123</v>
+        <v>227</v>
       </c>
       <c r="G747">
         <v>200</v>
@@ -22134,13 +22160,13 @@
         <v>697</v>
       </c>
       <c r="D748" t="s">
-        <v>323</v>
+        <v>205</v>
       </c>
       <c r="E748" t="s">
-        <v>324</v>
+        <v>206</v>
       </c>
       <c r="F748" t="s">
-        <v>324</v>
+        <v>206</v>
       </c>
       <c r="G748">
         <v>200</v>
@@ -22160,13 +22186,13 @@
         <v>697</v>
       </c>
       <c r="D749" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="E749" t="s">
-        <v>362</v>
+        <v>156</v>
       </c>
       <c r="F749" t="s">
-        <v>362</v>
+        <v>156</v>
       </c>
       <c r="G749">
         <v>200</v>
@@ -22186,13 +22212,13 @@
         <v>697</v>
       </c>
       <c r="D750" t="s">
-        <v>382</v>
+        <v>668</v>
       </c>
       <c r="E750" t="s">
-        <v>383</v>
+        <v>81</v>
       </c>
       <c r="F750" t="s">
-        <v>383</v>
+        <v>81</v>
       </c>
       <c r="G750">
         <v>200</v>
@@ -22201,30 +22227,30 @@
         <v>12</v>
       </c>
     </row>
-    <row r="751" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A751">
+    <row r="751" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A751" s="3">
         <v>750</v>
       </c>
-      <c r="B751" t="s">
-        <v>682</v>
-      </c>
-      <c r="C751" t="s">
-        <v>697</v>
-      </c>
-      <c r="D751" t="s">
-        <v>325</v>
-      </c>
-      <c r="E751" t="s">
-        <v>326</v>
-      </c>
-      <c r="F751" t="s">
-        <v>326</v>
-      </c>
-      <c r="G751">
-        <v>200</v>
-      </c>
-      <c r="H751" s="2" t="s">
-        <v>12</v>
+      <c r="B751" s="3" t="s">
+        <v>682</v>
+      </c>
+      <c r="C751" s="3" t="s">
+        <v>697</v>
+      </c>
+      <c r="D751" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E751" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="F751" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="G751" s="3">
+        <v>200</v>
+      </c>
+      <c r="H751" s="4" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="752" spans="1:8" x14ac:dyDescent="0.25">
@@ -22238,13 +22264,13 @@
         <v>697</v>
       </c>
       <c r="D752" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="E752" t="s">
-        <v>672</v>
+        <v>123</v>
       </c>
       <c r="F752" t="s">
-        <v>672</v>
+        <v>123</v>
       </c>
       <c r="G752">
         <v>200</v>
@@ -22264,13 +22290,13 @@
         <v>697</v>
       </c>
       <c r="D753" t="s">
-        <v>673</v>
+        <v>323</v>
       </c>
       <c r="E753" t="s">
-        <v>674</v>
+        <v>324</v>
       </c>
       <c r="F753" t="s">
-        <v>674</v>
+        <v>324</v>
       </c>
       <c r="G753">
         <v>200</v>
@@ -22290,13 +22316,13 @@
         <v>697</v>
       </c>
       <c r="D754" t="s">
-        <v>675</v>
+        <v>670</v>
       </c>
       <c r="E754" t="s">
-        <v>676</v>
+        <v>362</v>
       </c>
       <c r="F754" t="s">
-        <v>676</v>
+        <v>362</v>
       </c>
       <c r="G754">
         <v>200</v>
@@ -22316,13 +22342,13 @@
         <v>697</v>
       </c>
       <c r="D755" t="s">
-        <v>677</v>
+        <v>382</v>
       </c>
       <c r="E755" t="s">
-        <v>678</v>
+        <v>383</v>
       </c>
       <c r="F755" t="s">
-        <v>678</v>
+        <v>383</v>
       </c>
       <c r="G755">
         <v>200</v>
@@ -22342,13 +22368,13 @@
         <v>697</v>
       </c>
       <c r="D756" t="s">
-        <v>679</v>
+        <v>325</v>
       </c>
       <c r="E756" t="s">
-        <v>680</v>
+        <v>326</v>
       </c>
       <c r="F756" t="s">
-        <v>680</v>
+        <v>326</v>
       </c>
       <c r="G756">
         <v>200</v>
@@ -22368,13 +22394,13 @@
         <v>697</v>
       </c>
       <c r="D757" t="s">
-        <v>36</v>
+        <v>671</v>
       </c>
       <c r="E757" t="s">
-        <v>37</v>
+        <v>672</v>
       </c>
       <c r="F757" t="s">
-        <v>37</v>
+        <v>672</v>
       </c>
       <c r="G757">
         <v>200</v>
@@ -22394,13 +22420,13 @@
         <v>697</v>
       </c>
       <c r="D758" t="s">
-        <v>645</v>
+        <v>673</v>
       </c>
       <c r="E758" t="s">
-        <v>646</v>
+        <v>674</v>
       </c>
       <c r="F758" t="s">
-        <v>646</v>
+        <v>674</v>
       </c>
       <c r="G758">
         <v>200</v>
@@ -22420,19 +22446,260 @@
         <v>697</v>
       </c>
       <c r="D759" t="s">
+        <v>675</v>
+      </c>
+      <c r="E759" t="s">
+        <v>676</v>
+      </c>
+      <c r="F759" t="s">
+        <v>676</v>
+      </c>
+      <c r="G759">
+        <v>200</v>
+      </c>
+      <c r="H759" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="760" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A760">
+        <v>759</v>
+      </c>
+      <c r="B760" t="s">
+        <v>682</v>
+      </c>
+      <c r="C760" t="s">
+        <v>697</v>
+      </c>
+      <c r="D760" t="s">
+        <v>677</v>
+      </c>
+      <c r="E760" t="s">
+        <v>678</v>
+      </c>
+      <c r="F760" t="s">
+        <v>678</v>
+      </c>
+      <c r="G760">
+        <v>200</v>
+      </c>
+      <c r="H760" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="761" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A761">
+        <v>760</v>
+      </c>
+      <c r="B761" t="s">
+        <v>682</v>
+      </c>
+      <c r="C761" t="s">
+        <v>697</v>
+      </c>
+      <c r="D761" t="s">
+        <v>679</v>
+      </c>
+      <c r="E761" t="s">
+        <v>680</v>
+      </c>
+      <c r="F761" t="s">
+        <v>680</v>
+      </c>
+      <c r="G761">
+        <v>200</v>
+      </c>
+      <c r="H761" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="762" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A762">
+        <v>761</v>
+      </c>
+      <c r="B762" t="s">
+        <v>682</v>
+      </c>
+      <c r="C762" t="s">
+        <v>697</v>
+      </c>
+      <c r="D762" t="s">
+        <v>36</v>
+      </c>
+      <c r="E762" t="s">
+        <v>37</v>
+      </c>
+      <c r="F762" t="s">
+        <v>37</v>
+      </c>
+      <c r="G762">
+        <v>200</v>
+      </c>
+      <c r="H762" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="763" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A763">
+        <v>762</v>
+      </c>
+      <c r="B763" t="s">
+        <v>682</v>
+      </c>
+      <c r="C763" t="s">
+        <v>697</v>
+      </c>
+      <c r="D763" t="s">
+        <v>645</v>
+      </c>
+      <c r="E763" t="s">
+        <v>646</v>
+      </c>
+      <c r="F763" t="s">
+        <v>646</v>
+      </c>
+      <c r="G763">
+        <v>200</v>
+      </c>
+      <c r="H763" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="764" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A764">
+        <v>763</v>
+      </c>
+      <c r="B764" t="s">
+        <v>682</v>
+      </c>
+      <c r="C764" t="s">
+        <v>697</v>
+      </c>
+      <c r="D764" t="s">
         <v>681</v>
       </c>
-      <c r="E759" t="s">
+      <c r="E764" t="s">
         <v>648</v>
       </c>
-      <c r="F759" t="s">
+      <c r="F764" t="s">
         <v>648</v>
       </c>
-      <c r="G759">
-        <v>200</v>
-      </c>
-      <c r="H759" s="2" t="s">
-        <v>12</v>
+      <c r="G764">
+        <v>200</v>
+      </c>
+      <c r="H764" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="35" customWidth="1"/>
+    <col min="5" max="6" width="45" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>96</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>503</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E3" t="s">
+        <v>135</v>
+      </c>
+      <c r="F3" t="s">
+        <v>136</v>
+      </c>
+      <c r="G3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>750</v>
+      </c>
+      <c r="B4" t="s">
+        <v>682</v>
+      </c>
+      <c r="C4" t="s">
+        <v>697</v>
+      </c>
+      <c r="D4" t="s">
+        <v>134</v>
+      </c>
+      <c r="E4" t="s">
+        <v>135</v>
+      </c>
+      <c r="F4" t="s">
+        <v>136</v>
+      </c>
+      <c r="G4">
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>